<commit_message>
BOM changes (Alternates added)
</commit_message>
<xml_diff>
--- a/BOM/GTV3_Board/eSpark_BOM.xlsx
+++ b/BOM/GTV3_Board/eSpark_BOM.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25427"/>
-  <workbookPr codeName="ThisWorkbook"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr codeName="ThisWorkbook" defaultThemeVersion="153222"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\OliverStanton-WaterMonitor\BOM\GTV3_Board\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\Faizan\GitHub\OliverStanton-WaterMonitor\BOM\GTV3_Board\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{8DD7D7FE-7C6A-41D8-B9BE-2FE2CE9C28F7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="162913"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -30,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="937" uniqueCount="534">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="945" uniqueCount="540">
   <si>
     <t>Component list</t>
   </si>
@@ -1632,12 +1631,42 @@
   </si>
   <si>
     <t xml:space="preserve"> (GTV3)</t>
+  </si>
+  <si>
+    <t>T491A105K025AT</t>
+  </si>
+  <si>
+    <t>C123716</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Alternate added. </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="9"/>
+        <rFont val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Design change needed</t>
+    </r>
+  </si>
+  <si>
+    <t>SMBJ70A/TR13</t>
+  </si>
+  <si>
+    <t>C309982</t>
+  </si>
+  <si>
+    <t>Alternate added. Design change may not be needed. Needs to be confirmed</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
@@ -2149,7 +2178,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="101">
+  <cellXfs count="102">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1"/>
@@ -2431,6 +2460,9 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="17" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="6" borderId="16" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2773,32 +2805,32 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:T104"/>
-  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="2" max="2" width="3.140625" style="26" customWidth="1"/>
+    <col min="2" max="2" width="3.1796875" style="26" customWidth="1"/>
     <col min="3" max="3" width="18" style="26" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="27.42578125" customWidth="1"/>
-    <col min="5" max="5" width="30.85546875" customWidth="1"/>
-    <col min="6" max="6" width="22.28515625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="33.42578125" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="21.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="19.7109375" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="17.5703125" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="12" max="12" width="8.7109375" bestFit="1" customWidth="1"/>
-    <col min="13" max="13" width="17.28515625" bestFit="1" customWidth="1"/>
-    <col min="14" max="14" width="19.28515625" bestFit="1" customWidth="1"/>
-    <col min="15" max="15" width="10.28515625" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="17.7109375" bestFit="1" customWidth="1"/>
-    <col min="17" max="17" width="18.28515625" bestFit="1" customWidth="1"/>
-    <col min="18" max="18" width="16.5703125" bestFit="1" customWidth="1"/>
-    <col min="19" max="19" width="26.85546875" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27.453125" customWidth="1"/>
+    <col min="5" max="5" width="30.81640625" customWidth="1"/>
+    <col min="6" max="6" width="22.26953125" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="33.453125" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="21.54296875" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="19.7265625" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="17.54296875" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="10.7265625" bestFit="1" customWidth="1"/>
+    <col min="12" max="12" width="8.7265625" bestFit="1" customWidth="1"/>
+    <col min="13" max="13" width="17.26953125" bestFit="1" customWidth="1"/>
+    <col min="14" max="14" width="19.26953125" bestFit="1" customWidth="1"/>
+    <col min="15" max="15" width="10.26953125" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="17.7265625" bestFit="1" customWidth="1"/>
+    <col min="17" max="17" width="18.26953125" bestFit="1" customWidth="1"/>
+    <col min="18" max="18" width="16.54296875" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="26.81640625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A1" s="1"/>
       <c r="B1" s="20"/>
       <c r="C1" s="20"/>
@@ -2819,7 +2851,7 @@
       <c r="R1" s="93"/>
       <c r="S1" s="94"/>
     </row>
-    <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:19" ht="31.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="1"/>
       <c r="B2" s="21"/>
       <c r="C2" s="39"/>
@@ -2844,7 +2876,7 @@
       <c r="R2" s="4"/>
       <c r="S2" s="3"/>
     </row>
-    <row r="3" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A3" s="1"/>
       <c r="B3" s="22"/>
       <c r="C3" s="40"/>
@@ -2869,7 +2901,7 @@
       <c r="R3" s="5"/>
       <c r="S3" s="95"/>
     </row>
-    <row r="4" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A4" s="1"/>
       <c r="B4" s="22"/>
       <c r="C4" s="40"/>
@@ -2894,7 +2926,7 @@
       <c r="R4" s="6"/>
       <c r="S4" s="96"/>
     </row>
-    <row r="5" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A5" s="1"/>
       <c r="B5" s="22"/>
       <c r="C5" s="40"/>
@@ -2919,7 +2951,7 @@
       <c r="R5" s="6"/>
       <c r="S5" s="96"/>
     </row>
-    <row r="6" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A6" s="1"/>
       <c r="B6" s="23"/>
       <c r="C6" s="41"/>
@@ -2940,7 +2972,7 @@
       <c r="R6" s="6"/>
       <c r="S6" s="96"/>
     </row>
-    <row r="7" spans="1:19" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:19" x14ac:dyDescent="0.35">
       <c r="A7" s="1"/>
       <c r="B7" s="24"/>
       <c r="C7" s="42"/>
@@ -2961,7 +2993,7 @@
       <c r="R7" s="8"/>
       <c r="S7" s="96"/>
     </row>
-    <row r="8" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A8" s="1"/>
       <c r="B8" s="27"/>
       <c r="C8" s="43"/>
@@ -2982,7 +3014,7 @@
       <c r="R8" s="8"/>
       <c r="S8" s="96"/>
     </row>
-    <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A9" s="1"/>
       <c r="B9" s="30" t="s">
         <v>4</v>
@@ -3039,7 +3071,7 @@
         <v>410</v>
       </c>
     </row>
-    <row r="10" spans="1:19" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:19" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A10" s="1"/>
       <c r="B10" s="38">
         <f t="shared" ref="B10:B41" si="0">ROW(B10) - ROW($B$9)</f>
@@ -3095,7 +3127,7 @@
       <c r="R10" s="48"/>
       <c r="S10" s="49"/>
     </row>
-    <row r="11" spans="1:19" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:19" ht="60.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A11" s="1"/>
       <c r="B11" s="38">
         <f t="shared" si="0"/>
@@ -3151,7 +3183,7 @@
       <c r="R11" s="52"/>
       <c r="S11" s="53"/>
     </row>
-    <row r="12" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A12" s="1"/>
       <c r="B12" s="38">
         <f t="shared" si="0"/>
@@ -3207,7 +3239,7 @@
       <c r="R12" s="48"/>
       <c r="S12" s="48"/>
     </row>
-    <row r="13" spans="1:19" ht="48.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:19" ht="48.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A13" s="1"/>
       <c r="B13" s="38">
         <f t="shared" si="0"/>
@@ -3263,7 +3295,7 @@
       <c r="R13" s="52"/>
       <c r="S13" s="52"/>
     </row>
-    <row r="14" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A14" s="1"/>
       <c r="B14" s="38">
         <f t="shared" si="0"/>
@@ -3319,7 +3351,7 @@
       <c r="R14" s="48"/>
       <c r="S14" s="48"/>
     </row>
-    <row r="15" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A15" s="1"/>
       <c r="B15" s="38">
         <f t="shared" si="0"/>
@@ -3375,7 +3407,7 @@
       <c r="R15" s="52"/>
       <c r="S15" s="52"/>
     </row>
-    <row r="16" spans="1:19" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:19" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A16" s="1"/>
       <c r="B16" s="38">
         <f t="shared" si="0"/>
@@ -3396,11 +3428,15 @@
       <c r="G16" s="76" t="s">
         <v>195</v>
       </c>
-      <c r="H16" s="75"/>
+      <c r="H16" s="75" t="s">
+        <v>534</v>
+      </c>
       <c r="I16" s="75" t="s">
         <v>304</v>
       </c>
-      <c r="J16" s="75"/>
+      <c r="J16" s="75" t="s">
+        <v>535</v>
+      </c>
       <c r="K16" s="75" t="s">
         <v>343</v>
       </c>
@@ -3411,19 +3447,27 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="N16" s="75"/>
-      <c r="O16" s="75"/>
-      <c r="P16" s="77"/>
+      <c r="N16" s="75">
+        <v>10</v>
+      </c>
+      <c r="O16" s="101" t="s">
+        <v>417</v>
+      </c>
+      <c r="P16" s="77">
+        <v>0.187</v>
+      </c>
       <c r="Q16" s="77">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>1.87</v>
       </c>
       <c r="R16" s="83" t="s">
         <v>527</v>
       </c>
-      <c r="S16" s="78"/>
-    </row>
-    <row r="17" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S16" s="78" t="s">
+        <v>536</v>
+      </c>
+    </row>
+    <row r="17" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A17" s="1"/>
       <c r="B17" s="38">
         <f t="shared" si="0"/>
@@ -3479,7 +3523,7 @@
       <c r="R17" s="52"/>
       <c r="S17" s="52"/>
     </row>
-    <row r="18" spans="1:19" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A18" s="1"/>
       <c r="B18" s="38">
         <f t="shared" si="0"/>
@@ -3535,7 +3579,7 @@
       <c r="R18" s="48"/>
       <c r="S18" s="48"/>
     </row>
-    <row r="19" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A19" s="1"/>
       <c r="B19" s="38">
         <f t="shared" si="0"/>
@@ -3591,7 +3635,7 @@
       <c r="R19" s="52"/>
       <c r="S19" s="52"/>
     </row>
-    <row r="20" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A20" s="1"/>
       <c r="B20" s="38">
         <f t="shared" si="0"/>
@@ -3647,7 +3691,7 @@
       <c r="R20" s="48"/>
       <c r="S20" s="48"/>
     </row>
-    <row r="21" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A21" s="1"/>
       <c r="B21" s="38">
         <f t="shared" si="0"/>
@@ -3703,7 +3747,7 @@
       <c r="R21" s="52"/>
       <c r="S21" s="52"/>
     </row>
-    <row r="22" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A22" s="1"/>
       <c r="B22" s="38">
         <f t="shared" si="0"/>
@@ -3759,7 +3803,7 @@
       <c r="R22" s="48"/>
       <c r="S22" s="48"/>
     </row>
-    <row r="23" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A23" s="1"/>
       <c r="B23" s="38">
         <f t="shared" si="0"/>
@@ -3815,7 +3859,7 @@
       <c r="R23" s="52"/>
       <c r="S23" s="52"/>
     </row>
-    <row r="24" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A24" s="1"/>
       <c r="B24" s="38">
         <f t="shared" si="0"/>
@@ -3871,7 +3915,7 @@
       <c r="R24" s="48"/>
       <c r="S24" s="48"/>
     </row>
-    <row r="25" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A25" s="1"/>
       <c r="B25" s="38">
         <f t="shared" si="0"/>
@@ -3927,7 +3971,7 @@
       <c r="R25" s="52"/>
       <c r="S25" s="52"/>
     </row>
-    <row r="26" spans="1:19" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:19" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A26" s="1"/>
       <c r="B26" s="38">
         <f t="shared" si="0"/>
@@ -3983,7 +4027,7 @@
       <c r="R26" s="48"/>
       <c r="S26" s="48"/>
     </row>
-    <row r="27" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A27" s="1"/>
       <c r="B27" s="38">
         <f t="shared" si="0"/>
@@ -4039,7 +4083,7 @@
       <c r="R27" s="52"/>
       <c r="S27" s="52"/>
     </row>
-    <row r="28" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A28" s="1"/>
       <c r="B28" s="38">
         <f t="shared" si="0"/>
@@ -4093,7 +4137,7 @@
       <c r="R28" s="48"/>
       <c r="S28" s="48"/>
     </row>
-    <row r="29" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A29" s="1"/>
       <c r="B29" s="38">
         <f t="shared" si="0"/>
@@ -4149,7 +4193,7 @@
       <c r="R29" s="52"/>
       <c r="S29" s="52"/>
     </row>
-    <row r="30" spans="1:19" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:19" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A30" s="1"/>
       <c r="B30" s="38">
         <f t="shared" si="0"/>
@@ -4170,11 +4214,15 @@
       <c r="G30" s="76" t="s">
         <v>255</v>
       </c>
-      <c r="H30" s="75"/>
+      <c r="H30" s="75" t="s">
+        <v>537</v>
+      </c>
       <c r="I30" s="75" t="s">
         <v>308</v>
       </c>
-      <c r="J30" s="75"/>
+      <c r="J30" s="75" t="s">
+        <v>538</v>
+      </c>
       <c r="K30" s="75" t="s">
         <v>413</v>
       </c>
@@ -4185,19 +4233,27 @@
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="N30" s="75"/>
-      <c r="O30" s="75"/>
-      <c r="P30" s="77"/>
+      <c r="N30" s="75">
+        <v>10</v>
+      </c>
+      <c r="O30" s="101" t="s">
+        <v>417</v>
+      </c>
+      <c r="P30" s="77">
+        <v>6.9000000000000006E-2</v>
+      </c>
       <c r="Q30" s="77">
         <f t="shared" si="2"/>
-        <v>0</v>
+        <v>0.69000000000000006</v>
       </c>
       <c r="R30" s="83" t="s">
         <v>527</v>
       </c>
-      <c r="S30" s="78"/>
-    </row>
-    <row r="31" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="S30" s="78" t="s">
+        <v>539</v>
+      </c>
+    </row>
+    <row r="31" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A31" s="1"/>
       <c r="B31" s="38">
         <f t="shared" si="0"/>
@@ -4253,7 +4309,7 @@
       <c r="R31" s="52"/>
       <c r="S31" s="52"/>
     </row>
-    <row r="32" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A32" s="1"/>
       <c r="B32" s="38">
         <f t="shared" si="0"/>
@@ -4299,7 +4355,7 @@
       <c r="R32" s="48"/>
       <c r="S32" s="48"/>
     </row>
-    <row r="33" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A33" s="1"/>
       <c r="B33" s="38">
         <f t="shared" si="0"/>
@@ -4355,7 +4411,7 @@
       <c r="R33" s="52"/>
       <c r="S33" s="52"/>
     </row>
-    <row r="34" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A34" s="1"/>
       <c r="B34" s="38">
         <f t="shared" si="0"/>
@@ -4411,7 +4467,7 @@
       <c r="R34" s="48"/>
       <c r="S34" s="48"/>
     </row>
-    <row r="35" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A35" s="1"/>
       <c r="B35" s="38">
         <f t="shared" si="0"/>
@@ -4467,7 +4523,7 @@
       <c r="R35" s="52"/>
       <c r="S35" s="52"/>
     </row>
-    <row r="36" spans="1:19" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:19" ht="36.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A36" s="1"/>
       <c r="B36" s="38">
         <f t="shared" si="0"/>
@@ -4523,7 +4579,7 @@
       <c r="R36" s="48"/>
       <c r="S36" s="48"/>
     </row>
-    <row r="37" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A37" s="1"/>
       <c r="B37" s="38">
         <f t="shared" si="0"/>
@@ -4579,7 +4635,7 @@
       <c r="R37" s="52"/>
       <c r="S37" s="52"/>
     </row>
-    <row r="38" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A38" s="1"/>
       <c r="B38" s="38">
         <f t="shared" si="0"/>
@@ -4635,7 +4691,7 @@
       <c r="R38" s="48"/>
       <c r="S38" s="48"/>
     </row>
-    <row r="39" spans="1:19" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A39" s="1"/>
       <c r="B39" s="38">
         <f t="shared" si="0"/>
@@ -4691,7 +4747,7 @@
       <c r="R39" s="52"/>
       <c r="S39" s="52"/>
     </row>
-    <row r="40" spans="1:19" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:19" ht="36.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A40" s="1"/>
       <c r="B40" s="38">
         <f t="shared" si="0"/>
@@ -4747,7 +4803,7 @@
       <c r="R40" s="48"/>
       <c r="S40" s="48"/>
     </row>
-    <row r="41" spans="1:19" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A41" s="1"/>
       <c r="B41" s="38">
         <f t="shared" si="0"/>
@@ -4803,7 +4859,7 @@
       <c r="R41" s="52"/>
       <c r="S41" s="52"/>
     </row>
-    <row r="42" spans="1:19" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:19" ht="36.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A42" s="1"/>
       <c r="B42" s="38">
         <f t="shared" ref="B42:B73" si="3">ROW(B42) - ROW($B$9)</f>
@@ -4859,7 +4915,7 @@
       <c r="R42" s="48"/>
       <c r="S42" s="48"/>
     </row>
-    <row r="43" spans="1:19" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:19" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A43" s="1"/>
       <c r="B43" s="38">
         <f t="shared" si="3"/>
@@ -4915,7 +4971,7 @@
       <c r="R43" s="52"/>
       <c r="S43" s="52"/>
     </row>
-    <row r="44" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A44" s="1"/>
       <c r="B44" s="38">
         <f t="shared" si="3"/>
@@ -4971,7 +5027,7 @@
       <c r="R44" s="48"/>
       <c r="S44" s="48"/>
     </row>
-    <row r="45" spans="1:19" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:19" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A45" s="1"/>
       <c r="B45" s="38">
         <f t="shared" si="3"/>
@@ -5027,7 +5083,7 @@
       <c r="R45" s="52"/>
       <c r="S45" s="52"/>
     </row>
-    <row r="46" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A46" s="1"/>
       <c r="B46" s="38">
         <f t="shared" si="3"/>
@@ -5086,7 +5142,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="47" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A47" s="1"/>
       <c r="B47" s="38">
         <f t="shared" si="3"/>
@@ -5142,7 +5198,7 @@
       <c r="R47" s="52"/>
       <c r="S47" s="52"/>
     </row>
-    <row r="48" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A48" s="1"/>
       <c r="B48" s="38">
         <f t="shared" si="3"/>
@@ -5198,7 +5254,7 @@
       <c r="R48" s="48"/>
       <c r="S48" s="48"/>
     </row>
-    <row r="49" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A49" s="1"/>
       <c r="B49" s="38">
         <f t="shared" si="3"/>
@@ -5254,7 +5310,7 @@
       <c r="R49" s="52"/>
       <c r="S49" s="52"/>
     </row>
-    <row r="50" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A50" s="1"/>
       <c r="B50" s="38">
         <f t="shared" si="3"/>
@@ -5310,7 +5366,7 @@
       <c r="R50" s="48"/>
       <c r="S50" s="48"/>
     </row>
-    <row r="51" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A51" s="1"/>
       <c r="B51" s="38">
         <f t="shared" si="3"/>
@@ -5366,7 +5422,7 @@
       <c r="R51" s="52"/>
       <c r="S51" s="52"/>
     </row>
-    <row r="52" spans="1:19" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:19" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A52" s="1"/>
       <c r="B52" s="38">
         <f t="shared" si="3"/>
@@ -5422,7 +5478,7 @@
       <c r="R52" s="48"/>
       <c r="S52" s="48"/>
     </row>
-    <row r="53" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A53" s="1"/>
       <c r="B53" s="38">
         <f t="shared" si="3"/>
@@ -5478,7 +5534,7 @@
       <c r="R53" s="52"/>
       <c r="S53" s="52"/>
     </row>
-    <row r="54" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A54" s="1"/>
       <c r="B54" s="38">
         <f t="shared" si="3"/>
@@ -5532,7 +5588,7 @@
       <c r="R54" s="48"/>
       <c r="S54" s="48"/>
     </row>
-    <row r="55" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A55" s="1"/>
       <c r="B55" s="38">
         <f t="shared" si="3"/>
@@ -5588,7 +5644,7 @@
       <c r="R55" s="52"/>
       <c r="S55" s="52"/>
     </row>
-    <row r="56" spans="1:19" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:19" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A56" s="1"/>
       <c r="B56" s="38">
         <f t="shared" si="3"/>
@@ -5642,7 +5698,7 @@
       <c r="R56" s="48"/>
       <c r="S56" s="48"/>
     </row>
-    <row r="57" spans="1:19" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:19" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A57" s="1"/>
       <c r="B57" s="38">
         <f t="shared" si="3"/>
@@ -5698,7 +5754,7 @@
       <c r="R57" s="52"/>
       <c r="S57" s="52"/>
     </row>
-    <row r="58" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A58" s="1"/>
       <c r="B58" s="38">
         <f t="shared" si="3"/>
@@ -5754,7 +5810,7 @@
       <c r="R58" s="48"/>
       <c r="S58" s="48"/>
     </row>
-    <row r="59" spans="1:19" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:19" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A59" s="1"/>
       <c r="B59" s="38">
         <f t="shared" si="3"/>
@@ -5810,7 +5866,7 @@
       <c r="R59" s="52"/>
       <c r="S59" s="52"/>
     </row>
-    <row r="60" spans="1:19" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:19" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A60" s="1"/>
       <c r="B60" s="38">
         <f t="shared" si="3"/>
@@ -5866,7 +5922,7 @@
       <c r="R60" s="48"/>
       <c r="S60" s="48"/>
     </row>
-    <row r="61" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A61" s="1"/>
       <c r="B61" s="38">
         <f t="shared" si="3"/>
@@ -5920,7 +5976,7 @@
       <c r="R61" s="52"/>
       <c r="S61" s="52"/>
     </row>
-    <row r="62" spans="1:19" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:19" ht="36.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A62" s="1"/>
       <c r="B62" s="38">
         <f t="shared" si="3"/>
@@ -5976,7 +6032,7 @@
       <c r="R62" s="48"/>
       <c r="S62" s="48"/>
     </row>
-    <row r="63" spans="1:19" ht="60.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:19" ht="60.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A63" s="1"/>
       <c r="B63" s="38">
         <f t="shared" si="3"/>
@@ -6032,7 +6088,7 @@
       <c r="R63" s="52"/>
       <c r="S63" s="52"/>
     </row>
-    <row r="64" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A64" s="1"/>
       <c r="B64" s="38">
         <f t="shared" si="3"/>
@@ -6088,7 +6144,7 @@
       <c r="R64" s="48"/>
       <c r="S64" s="48"/>
     </row>
-    <row r="65" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A65" s="1"/>
       <c r="B65" s="38">
         <f t="shared" si="3"/>
@@ -6142,7 +6198,7 @@
       <c r="R65" s="52"/>
       <c r="S65" s="52"/>
     </row>
-    <row r="66" spans="1:19" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:19" ht="36.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A66" s="1"/>
       <c r="B66" s="38">
         <f t="shared" si="3"/>
@@ -6198,7 +6254,7 @@
       <c r="R66" s="48"/>
       <c r="S66" s="48"/>
     </row>
-    <row r="67" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A67" s="1"/>
       <c r="B67" s="38">
         <f t="shared" si="3"/>
@@ -6254,7 +6310,7 @@
       <c r="R67" s="52"/>
       <c r="S67" s="52"/>
     </row>
-    <row r="68" spans="1:19" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A68" s="1"/>
       <c r="B68" s="38">
         <f t="shared" si="3"/>
@@ -6310,7 +6366,7 @@
       <c r="R68" s="48"/>
       <c r="S68" s="48"/>
     </row>
-    <row r="69" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A69" s="1"/>
       <c r="B69" s="38">
         <f t="shared" si="3"/>
@@ -6366,7 +6422,7 @@
       <c r="R69" s="52"/>
       <c r="S69" s="52"/>
     </row>
-    <row r="70" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A70" s="1"/>
       <c r="B70" s="38">
         <f t="shared" si="3"/>
@@ -6422,7 +6478,7 @@
       <c r="R70" s="48"/>
       <c r="S70" s="48"/>
     </row>
-    <row r="71" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A71" s="1"/>
       <c r="B71" s="38">
         <f t="shared" si="3"/>
@@ -6478,7 +6534,7 @@
       <c r="R71" s="52"/>
       <c r="S71" s="52"/>
     </row>
-    <row r="72" spans="1:19" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:19" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A72" s="1"/>
       <c r="B72" s="38">
         <f t="shared" si="3"/>
@@ -6534,7 +6590,7 @@
       <c r="R72" s="48"/>
       <c r="S72" s="48"/>
     </row>
-    <row r="73" spans="1:19" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:19" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A73" s="1"/>
       <c r="B73" s="38">
         <f t="shared" si="3"/>
@@ -6590,7 +6646,7 @@
       <c r="R73" s="52"/>
       <c r="S73" s="52"/>
     </row>
-    <row r="74" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A74" s="1"/>
       <c r="B74" s="38">
         <f t="shared" ref="B74:B101" si="4">ROW(B74) - ROW($B$9)</f>
@@ -6646,7 +6702,7 @@
       <c r="R74" s="90"/>
       <c r="S74" s="48"/>
     </row>
-    <row r="75" spans="1:19" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:19" ht="36.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A75" s="1"/>
       <c r="B75" s="38">
         <f t="shared" si="4"/>
@@ -6702,7 +6758,7 @@
       <c r="R75" s="52"/>
       <c r="S75" s="52"/>
     </row>
-    <row r="76" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A76" s="1"/>
       <c r="B76" s="38">
         <f t="shared" si="4"/>
@@ -6758,7 +6814,7 @@
       <c r="R76" s="48"/>
       <c r="S76" s="48"/>
     </row>
-    <row r="77" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A77" s="1"/>
       <c r="B77" s="38">
         <f t="shared" si="4"/>
@@ -6814,7 +6870,7 @@
       <c r="R77" s="52"/>
       <c r="S77" s="52"/>
     </row>
-    <row r="78" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A78" s="1"/>
       <c r="B78" s="38">
         <f t="shared" si="4"/>
@@ -6870,7 +6926,7 @@
       <c r="R78" s="48"/>
       <c r="S78" s="48"/>
     </row>
-    <row r="79" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A79" s="1"/>
       <c r="B79" s="38">
         <f t="shared" si="4"/>
@@ -6926,7 +6982,7 @@
       <c r="R79" s="52"/>
       <c r="S79" s="52"/>
     </row>
-    <row r="80" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A80" s="1"/>
       <c r="B80" s="38">
         <f t="shared" si="4"/>
@@ -6982,7 +7038,7 @@
       <c r="R80" s="48"/>
       <c r="S80" s="48"/>
     </row>
-    <row r="81" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A81" s="1"/>
       <c r="B81" s="38">
         <f t="shared" si="4"/>
@@ -7038,7 +7094,7 @@
       <c r="R81" s="48"/>
       <c r="S81" s="48"/>
     </row>
-    <row r="82" spans="1:20" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:20" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A82" s="1"/>
       <c r="B82" s="38">
         <f t="shared" si="4"/>
@@ -7094,7 +7150,7 @@
       <c r="R82" s="52"/>
       <c r="S82" s="52"/>
     </row>
-    <row r="83" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A83" s="1"/>
       <c r="B83" s="38">
         <f t="shared" si="4"/>
@@ -7150,7 +7206,7 @@
       <c r="R83" s="48"/>
       <c r="S83" s="48"/>
     </row>
-    <row r="84" spans="1:20" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:20" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A84" s="1"/>
       <c r="B84" s="38">
         <f t="shared" si="4"/>
@@ -7206,7 +7262,7 @@
       <c r="R84" s="52"/>
       <c r="S84" s="52"/>
     </row>
-    <row r="85" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A85" s="1"/>
       <c r="B85" s="38">
         <f t="shared" si="4"/>
@@ -7262,7 +7318,7 @@
       <c r="R85" s="48"/>
       <c r="S85" s="48"/>
     </row>
-    <row r="86" spans="1:20" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:20" ht="36.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A86" s="1"/>
       <c r="B86" s="38">
         <f t="shared" si="4"/>
@@ -7321,7 +7377,7 @@
         <v>413</v>
       </c>
     </row>
-    <row r="87" spans="1:20" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A87" s="1"/>
       <c r="B87" s="38">
         <f t="shared" si="4"/>
@@ -7377,7 +7433,7 @@
       <c r="R87" s="48"/>
       <c r="S87" s="48"/>
     </row>
-    <row r="88" spans="1:20" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:20" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A88" s="1"/>
       <c r="B88" s="38">
         <f t="shared" si="4"/>
@@ -7436,7 +7492,7 @@
       <c r="S88" s="68"/>
       <c r="T88" s="79"/>
     </row>
-    <row r="89" spans="1:20" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:20" ht="36.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A89" s="1"/>
       <c r="B89" s="38">
         <f t="shared" si="4"/>
@@ -7492,7 +7548,7 @@
       <c r="R89" s="48"/>
       <c r="S89" s="48"/>
     </row>
-    <row r="90" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A90" s="1"/>
       <c r="B90" s="38">
         <f t="shared" si="4"/>
@@ -7548,7 +7604,7 @@
       <c r="R90" s="52"/>
       <c r="S90" s="52"/>
     </row>
-    <row r="91" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A91" s="1"/>
       <c r="B91" s="38">
         <f t="shared" si="4"/>
@@ -7604,7 +7660,7 @@
       <c r="R91" s="48"/>
       <c r="S91" s="48"/>
     </row>
-    <row r="92" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A92" s="1"/>
       <c r="B92" s="38">
         <f t="shared" si="4"/>
@@ -7654,7 +7710,7 @@
       <c r="R92" s="68"/>
       <c r="S92" s="68"/>
     </row>
-    <row r="93" spans="1:20" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:20" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A93" s="1"/>
       <c r="B93" s="38">
         <f t="shared" si="4"/>
@@ -7702,7 +7758,7 @@
       <c r="R93" s="78"/>
       <c r="S93" s="78"/>
     </row>
-    <row r="94" spans="1:20" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:20" ht="24.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A94" s="1"/>
       <c r="B94" s="38">
         <f t="shared" si="4"/>
@@ -7758,7 +7814,7 @@
       <c r="R94" s="52"/>
       <c r="S94" s="52"/>
     </row>
-    <row r="95" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A95" s="1"/>
       <c r="B95" s="38">
         <f t="shared" si="4"/>
@@ -7814,7 +7870,7 @@
       <c r="R95" s="48"/>
       <c r="S95" s="48"/>
     </row>
-    <row r="96" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:20" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A96" s="1"/>
       <c r="B96" s="38">
         <f t="shared" si="4"/>
@@ -7870,7 +7926,7 @@
       <c r="R96" s="52"/>
       <c r="S96" s="52"/>
     </row>
-    <row r="97" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A97" s="1"/>
       <c r="B97" s="38">
         <f t="shared" si="4"/>
@@ -7926,7 +7982,7 @@
       <c r="R97" s="48"/>
       <c r="S97" s="48"/>
     </row>
-    <row r="98" spans="1:19" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:19" ht="15" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A98" s="1"/>
       <c r="B98" s="38">
         <f t="shared" si="4"/>
@@ -7982,7 +8038,7 @@
       <c r="R98" s="52"/>
       <c r="S98" s="52"/>
     </row>
-    <row r="99" spans="1:19" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:19" ht="36.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A99" s="1"/>
       <c r="B99" s="38">
         <f t="shared" si="4"/>
@@ -8028,7 +8084,7 @@
       </c>
       <c r="S99" s="78"/>
     </row>
-    <row r="100" spans="1:19" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:19" ht="36.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A100" s="1"/>
       <c r="B100" s="38">
         <f t="shared" si="4"/>
@@ -8084,7 +8140,7 @@
       <c r="R100" s="52"/>
       <c r="S100" s="52"/>
     </row>
-    <row r="101" spans="1:19" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:19" ht="36.5" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A101" s="1"/>
       <c r="B101" s="38">
         <f t="shared" si="4"/>
@@ -8140,7 +8196,7 @@
       <c r="R101" s="48"/>
       <c r="S101" s="48"/>
     </row>
-    <row r="102" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:19" ht="19" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A102" s="1"/>
       <c r="B102" s="33"/>
       <c r="C102" s="44"/>
@@ -8161,12 +8217,12 @@
       <c r="P102" s="92"/>
       <c r="Q102" s="80">
         <f>SUM(Q10:Q101)</f>
-        <v>631.50729999999987</v>
+        <v>634.06729999999993</v>
       </c>
       <c r="R102" s="97"/>
       <c r="S102" s="98"/>
     </row>
-    <row r="103" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:19" ht="19" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A103" s="1"/>
       <c r="B103" s="25"/>
       <c r="C103" s="45"/>
@@ -8187,12 +8243,12 @@
       <c r="P103" s="92"/>
       <c r="Q103" s="81">
         <f>Q102/5</f>
-        <v>126.30145999999998</v>
+        <v>126.81345999999999</v>
       </c>
       <c r="R103" s="99"/>
       <c r="S103" s="100"/>
     </row>
-    <row r="104" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:19" ht="19" thickBot="1" x14ac:dyDescent="0.4">
       <c r="N104" s="91" t="s">
         <v>530</v>
       </c>
@@ -8212,93 +8268,95 @@
     <mergeCell ref="N103:P103"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="O10" r:id="rId1" xr:uid="{2E7196B7-17EB-4A3A-BBBE-F20142496754}"/>
-    <hyperlink ref="O11" r:id="rId2" xr:uid="{24227A28-30E3-4A7D-ACC9-83A1D87F2814}"/>
-    <hyperlink ref="O12" r:id="rId3" xr:uid="{FE1BDC2E-67C0-4AE9-81C8-6B7625F73009}"/>
-    <hyperlink ref="O13" r:id="rId4" xr:uid="{D8DC4BD8-BB31-4475-87D9-77DFEAD6280B}"/>
-    <hyperlink ref="O14" r:id="rId5" xr:uid="{246E2BF4-9826-45DD-ADA8-DF23CD0CC4F2}"/>
-    <hyperlink ref="O15" r:id="rId6" xr:uid="{D5F16A6B-52BB-43D6-8702-EA0BF946361C}"/>
-    <hyperlink ref="O17" r:id="rId7" xr:uid="{5C3ECBEF-9B20-4C72-85C5-B4210DC008FD}"/>
-    <hyperlink ref="O18" r:id="rId8" xr:uid="{DF660B85-FEA9-4E78-AAB7-56C6430CEBC0}"/>
-    <hyperlink ref="O19" r:id="rId9" xr:uid="{5D833557-62FB-4318-A648-FECDB3290C49}"/>
-    <hyperlink ref="O20" r:id="rId10" xr:uid="{A77EE9E0-3F15-4656-8237-A38358068CB4}"/>
-    <hyperlink ref="O21" r:id="rId11" xr:uid="{F5EBB4F2-5D4F-4F10-9A5D-BE0AC22B0A3F}"/>
-    <hyperlink ref="O22" r:id="rId12" xr:uid="{B9728DA4-DACA-488C-9A7D-342492186C6F}"/>
-    <hyperlink ref="O23" r:id="rId13" xr:uid="{0B123D99-8953-4429-A15F-E310BEC5E7FA}"/>
-    <hyperlink ref="O25" r:id="rId14" xr:uid="{B834ADAC-D117-49B4-AD7D-D27ABB605326}"/>
-    <hyperlink ref="O27" r:id="rId15" xr:uid="{A9100168-CD31-4482-9E96-2622C02A8427}"/>
-    <hyperlink ref="O36" r:id="rId16" xr:uid="{E1F1180A-2EF4-48E2-BF4F-12BEB776CA80}"/>
-    <hyperlink ref="O37" r:id="rId17" xr:uid="{C73A8BCC-86F8-4109-9AA9-B8D7DCE5EDCC}"/>
-    <hyperlink ref="O38" r:id="rId18" xr:uid="{16ECCE03-F673-4B2F-AA89-98A78F1A010A}"/>
-    <hyperlink ref="O40" r:id="rId19" xr:uid="{3D33F6C6-EBE5-436A-B4B0-9AA6044319D4}"/>
-    <hyperlink ref="O41" r:id="rId20" xr:uid="{DB56F5A6-D7AA-4B76-8F79-4DAB313B8056}"/>
-    <hyperlink ref="O42" r:id="rId21" xr:uid="{6EBA3756-8023-4DF9-8FB1-B45C9480F54D}"/>
-    <hyperlink ref="O44" r:id="rId22" xr:uid="{6D9D8028-81E4-4B1C-86B4-78EE5E55E0EB}"/>
-    <hyperlink ref="O45" r:id="rId23" xr:uid="{7D83DD86-CFE0-4253-8E76-35ABC5EA9FF9}"/>
-    <hyperlink ref="O52" r:id="rId24" xr:uid="{24B8AC9E-A4A4-4B9C-95D4-DF0D6051993E}"/>
-    <hyperlink ref="O54" r:id="rId25" xr:uid="{BE8193C0-1672-4B36-84FB-0231DA27A220}"/>
-    <hyperlink ref="O56" r:id="rId26" xr:uid="{85D9A402-8D38-44F2-B1CF-1609D072A63F}"/>
-    <hyperlink ref="O57" r:id="rId27" xr:uid="{40079AA9-5725-4514-9EE1-DE8FE129C438}"/>
-    <hyperlink ref="O58" r:id="rId28" xr:uid="{E2D69BC1-8723-468A-ADB6-F830AADF30C1}"/>
-    <hyperlink ref="O59" r:id="rId29" xr:uid="{CFE6F118-E798-4E0B-A0FA-D24BF1A27CF2}"/>
-    <hyperlink ref="O60" r:id="rId30" xr:uid="{376CDFD1-8D98-4D6F-9D9A-4DE42C6E03FB}"/>
-    <hyperlink ref="O61" r:id="rId31" xr:uid="{9DB40F78-1BDD-431D-95AE-C3066D199D75}"/>
-    <hyperlink ref="O62" r:id="rId32" xr:uid="{E0245546-F21A-4E75-B510-20365CA0EAEB}"/>
-    <hyperlink ref="O63" r:id="rId33" xr:uid="{808035A3-95B3-4248-983D-817557948EFB}"/>
-    <hyperlink ref="O64" r:id="rId34" xr:uid="{8A6D7048-03EF-4773-85D1-8F679B58BDAB}"/>
-    <hyperlink ref="O65" r:id="rId35" xr:uid="{614B8F76-BE4A-44CB-9C26-FF296675C3D7}"/>
-    <hyperlink ref="O66" r:id="rId36" xr:uid="{C518E7DB-4F17-4335-AC87-6250C5BC9693}"/>
-    <hyperlink ref="O68" r:id="rId37" xr:uid="{3043F893-14F3-4F75-A2C8-F9D922DC4D7B}"/>
-    <hyperlink ref="O69" r:id="rId38" xr:uid="{7BB98244-A23C-43F1-A7BD-4270CB605E86}"/>
-    <hyperlink ref="O70" r:id="rId39" xr:uid="{5950984E-7074-45F7-A52C-EDBB04B052A8}"/>
-    <hyperlink ref="O71" r:id="rId40" xr:uid="{D384A66B-1AB5-4A86-B1C5-6C36C800FBA3}"/>
-    <hyperlink ref="O72" r:id="rId41" xr:uid="{D416CA2F-3DBF-4BB5-91E4-50A4CCB83ABC}"/>
-    <hyperlink ref="O73" r:id="rId42" xr:uid="{312B558E-0D5B-4126-B5AB-4B06E093259E}"/>
-    <hyperlink ref="O75" r:id="rId43" xr:uid="{A83E4AFA-DC3C-4F6F-9BA8-8CCB97C53575}"/>
-    <hyperlink ref="O76" r:id="rId44" xr:uid="{5B9E54E0-D624-4CC8-8CBE-30254539C315}"/>
-    <hyperlink ref="O77" r:id="rId45" xr:uid="{6E1A2172-8A3F-4184-B677-FF40B43491AA}"/>
-    <hyperlink ref="O79" r:id="rId46" xr:uid="{93508975-457A-495D-8C37-E21E004DA0FE}"/>
-    <hyperlink ref="O80" r:id="rId47" xr:uid="{5214ED38-8616-4700-926D-3D34D13FEF40}"/>
-    <hyperlink ref="O81" r:id="rId48" xr:uid="{E4237223-8C39-4258-81BA-1615D2399A7B}"/>
-    <hyperlink ref="O82" r:id="rId49" xr:uid="{E11A4332-E6EA-43AB-B359-BCC6F3C401C4}"/>
-    <hyperlink ref="O84" r:id="rId50" xr:uid="{885B123B-5528-4DCE-9DC8-6F335281E245}"/>
-    <hyperlink ref="O87" r:id="rId51" xr:uid="{D2BCBDF9-A74C-4A3A-8625-58A6D16FA728}"/>
-    <hyperlink ref="O90" r:id="rId52" xr:uid="{C1025EBE-2B9B-4F82-8913-94E8D4B70C8C}"/>
-    <hyperlink ref="O91" r:id="rId53" xr:uid="{109E99DF-E179-48CA-A871-3FA35403FA40}"/>
-    <hyperlink ref="O95" r:id="rId54" xr:uid="{63489A4D-1105-4254-8892-B747CA8BE6D3}"/>
-    <hyperlink ref="O96" r:id="rId55" xr:uid="{205C45C9-5385-4B71-82F6-CB22EFEC03BC}"/>
-    <hyperlink ref="O97" r:id="rId56" xr:uid="{A10C0B1A-0547-4AC0-AECA-204CEC50389E}"/>
-    <hyperlink ref="O98" r:id="rId57" xr:uid="{35539995-C6B5-49E5-A00F-C4B539647ACB}"/>
-    <hyperlink ref="O100" r:id="rId58" xr:uid="{7BEA1386-CA7B-4873-84C1-67E96EA97C79}"/>
-    <hyperlink ref="O101" r:id="rId59" xr:uid="{13129D58-7A45-4DD5-AC01-7C42CB68552D}"/>
-    <hyperlink ref="O24" r:id="rId60" xr:uid="{15FF2D2C-F071-49A7-B625-CBE8AA250DF5}"/>
-    <hyperlink ref="O26" r:id="rId61" xr:uid="{296ADE2F-94C6-475B-86AF-821FD35EABB0}"/>
-    <hyperlink ref="O28" r:id="rId62" xr:uid="{F7A2A4B1-F69F-4744-BB3C-5C200EC38EA3}"/>
-    <hyperlink ref="O29" r:id="rId63" xr:uid="{83E2D456-8F59-4B57-A870-65274D6BCFFA}"/>
-    <hyperlink ref="O31" r:id="rId64" xr:uid="{A3BBB744-9B26-4CE1-9889-17E03774FE31}"/>
-    <hyperlink ref="O39" r:id="rId65" xr:uid="{58AEC90B-9C24-4FA1-AA38-1B8769D8BB10}"/>
-    <hyperlink ref="O48" r:id="rId66" xr:uid="{4890ACA3-FED0-4E73-9982-AA6245652B0C}"/>
-    <hyperlink ref="O47" r:id="rId67" xr:uid="{BD6A81E4-6E68-4A59-918A-E9410103558D}"/>
-    <hyperlink ref="O50" r:id="rId68" xr:uid="{9B3EA203-3D3F-4532-9D94-2F69C0008A4C}"/>
-    <hyperlink ref="O51" r:id="rId69" xr:uid="{F590DF7E-371F-4B84-907D-3BC02339C38C}"/>
-    <hyperlink ref="O53" r:id="rId70" xr:uid="{1DDC40AA-C78A-46B5-88ED-BC2B5B1C3144}"/>
-    <hyperlink ref="O55" r:id="rId71" xr:uid="{FDA2E76A-BC42-4AB9-871C-1D222BC8C85D}"/>
-    <hyperlink ref="O67" r:id="rId72" xr:uid="{396F44C7-85C4-4377-9EAB-0335589BB424}"/>
-    <hyperlink ref="O83" r:id="rId73" xr:uid="{7371F9D6-A4BF-4392-8175-E9F1945CB6A6}"/>
-    <hyperlink ref="O85" r:id="rId74" xr:uid="{771D1A85-11B5-407A-BCFB-293D31484E38}"/>
-    <hyperlink ref="O43" r:id="rId75" xr:uid="{430AC511-348E-4F5D-BF43-D38C5AD2ACDB}"/>
-    <hyperlink ref="O49" r:id="rId76" xr:uid="{60D3E071-83F1-4E3E-B99A-CF0DAB7C0848}"/>
-    <hyperlink ref="O74" r:id="rId77" xr:uid="{DDB3781D-CC67-4B9E-8A92-8B0D42E9ADD9}"/>
-    <hyperlink ref="O78" r:id="rId78" xr:uid="{C5625C77-072D-4075-87C6-94DA55FC1A0E}"/>
-    <hyperlink ref="O89" r:id="rId79" xr:uid="{68211B1F-D1FA-4BB4-B9AA-AD1AC06623A0}"/>
-    <hyperlink ref="O94" r:id="rId80" xr:uid="{E93B1DAB-AF05-4E07-8DD3-14AFCDF08ABE}"/>
-    <hyperlink ref="O33" r:id="rId81" xr:uid="{0249B8C0-EAE9-4590-9A86-81848E63EDB2}"/>
-    <hyperlink ref="O34" r:id="rId82" xr:uid="{ED947ABD-8BE1-4E62-8651-5924B800CF3D}"/>
-    <hyperlink ref="O35" r:id="rId83" xr:uid="{8AFB85E6-CCEB-4153-966B-2274E3C5FBE5}"/>
-    <hyperlink ref="O88" r:id="rId84" xr:uid="{508DF2DE-64C1-482F-9133-86D081915FC1}"/>
+    <hyperlink ref="O10" r:id="rId1"/>
+    <hyperlink ref="O11" r:id="rId2"/>
+    <hyperlink ref="O12" r:id="rId3"/>
+    <hyperlink ref="O13" r:id="rId4"/>
+    <hyperlink ref="O14" r:id="rId5"/>
+    <hyperlink ref="O15" r:id="rId6"/>
+    <hyperlink ref="O17" r:id="rId7"/>
+    <hyperlink ref="O18" r:id="rId8"/>
+    <hyperlink ref="O19" r:id="rId9"/>
+    <hyperlink ref="O20" r:id="rId10"/>
+    <hyperlink ref="O21" r:id="rId11"/>
+    <hyperlink ref="O22" r:id="rId12"/>
+    <hyperlink ref="O23" r:id="rId13"/>
+    <hyperlink ref="O25" r:id="rId14"/>
+    <hyperlink ref="O27" r:id="rId15"/>
+    <hyperlink ref="O36" r:id="rId16"/>
+    <hyperlink ref="O37" r:id="rId17"/>
+    <hyperlink ref="O38" r:id="rId18"/>
+    <hyperlink ref="O40" r:id="rId19"/>
+    <hyperlink ref="O41" r:id="rId20"/>
+    <hyperlink ref="O42" r:id="rId21"/>
+    <hyperlink ref="O44" r:id="rId22"/>
+    <hyperlink ref="O45" r:id="rId23"/>
+    <hyperlink ref="O52" r:id="rId24"/>
+    <hyperlink ref="O54" r:id="rId25"/>
+    <hyperlink ref="O56" r:id="rId26"/>
+    <hyperlink ref="O57" r:id="rId27"/>
+    <hyperlink ref="O58" r:id="rId28"/>
+    <hyperlink ref="O59" r:id="rId29"/>
+    <hyperlink ref="O60" r:id="rId30"/>
+    <hyperlink ref="O61" r:id="rId31"/>
+    <hyperlink ref="O62" r:id="rId32"/>
+    <hyperlink ref="O63" r:id="rId33"/>
+    <hyperlink ref="O64" r:id="rId34"/>
+    <hyperlink ref="O65" r:id="rId35"/>
+    <hyperlink ref="O66" r:id="rId36"/>
+    <hyperlink ref="O68" r:id="rId37"/>
+    <hyperlink ref="O69" r:id="rId38"/>
+    <hyperlink ref="O70" r:id="rId39"/>
+    <hyperlink ref="O71" r:id="rId40"/>
+    <hyperlink ref="O72" r:id="rId41"/>
+    <hyperlink ref="O73" r:id="rId42"/>
+    <hyperlink ref="O75" r:id="rId43"/>
+    <hyperlink ref="O76" r:id="rId44"/>
+    <hyperlink ref="O77" r:id="rId45"/>
+    <hyperlink ref="O79" r:id="rId46"/>
+    <hyperlink ref="O80" r:id="rId47"/>
+    <hyperlink ref="O81" r:id="rId48"/>
+    <hyperlink ref="O82" r:id="rId49"/>
+    <hyperlink ref="O84" r:id="rId50"/>
+    <hyperlink ref="O87" r:id="rId51"/>
+    <hyperlink ref="O90" r:id="rId52"/>
+    <hyperlink ref="O91" r:id="rId53"/>
+    <hyperlink ref="O95" r:id="rId54"/>
+    <hyperlink ref="O96" r:id="rId55"/>
+    <hyperlink ref="O97" r:id="rId56"/>
+    <hyperlink ref="O98" r:id="rId57"/>
+    <hyperlink ref="O100" r:id="rId58"/>
+    <hyperlink ref="O101" r:id="rId59"/>
+    <hyperlink ref="O24" r:id="rId60"/>
+    <hyperlink ref="O26" r:id="rId61"/>
+    <hyperlink ref="O28" r:id="rId62"/>
+    <hyperlink ref="O29" r:id="rId63"/>
+    <hyperlink ref="O31" r:id="rId64"/>
+    <hyperlink ref="O39" r:id="rId65"/>
+    <hyperlink ref="O48" r:id="rId66"/>
+    <hyperlink ref="O47" r:id="rId67"/>
+    <hyperlink ref="O50" r:id="rId68"/>
+    <hyperlink ref="O51" r:id="rId69"/>
+    <hyperlink ref="O53" r:id="rId70"/>
+    <hyperlink ref="O55" r:id="rId71"/>
+    <hyperlink ref="O67" r:id="rId72"/>
+    <hyperlink ref="O83" r:id="rId73"/>
+    <hyperlink ref="O85" r:id="rId74"/>
+    <hyperlink ref="O43" r:id="rId75"/>
+    <hyperlink ref="O49" r:id="rId76"/>
+    <hyperlink ref="O74" r:id="rId77"/>
+    <hyperlink ref="O78" r:id="rId78"/>
+    <hyperlink ref="O89" r:id="rId79"/>
+    <hyperlink ref="O94" r:id="rId80"/>
+    <hyperlink ref="O33" r:id="rId81"/>
+    <hyperlink ref="O34" r:id="rId82"/>
+    <hyperlink ref="O35" r:id="rId83"/>
+    <hyperlink ref="O88" r:id="rId84"/>
+    <hyperlink ref="O16" r:id="rId85"/>
+    <hyperlink ref="O30" r:id="rId86"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="9" orientation="portrait" r:id="rId85"/>
-  <drawing r:id="rId86"/>
+  <pageSetup paperSize="9" orientation="portrait" r:id="rId87"/>
+  <drawing r:id="rId88"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Superb Automation quotes updated in GTV3 BOM
</commit_message>
<xml_diff>
--- a/BOM/GTV3_Board/eSpark_BOM.xlsx
+++ b/BOM/GTV3_Board/eSpark_BOM.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="25427"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
   <workbookPr codeName="ThisWorkbook"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\GitHub\OliverStanton-WaterMonitor\BOM\GTV3_Board\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Faizan\GitHub\OliverStanton-WaterMonitor\BOM\GTV3_Board\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{29721828-455E-4D8A-81C6-4B1D2E0033E3}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-5265" yWindow="2205" windowWidth="11790" windowHeight="15360" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-5265" yWindow="2205" windowWidth="11790" windowHeight="15360"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="181029"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
       <xcalcf:calcFeatures>
@@ -30,7 +29,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="951" uniqueCount="545">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="952" uniqueCount="543">
   <si>
     <t>Component list</t>
   </si>
@@ -1584,12 +1583,6 @@
   </si>
   <si>
     <t>C441238</t>
-  </si>
-  <si>
-    <t>Aliexpress</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Is part ki Shipping Cost Add ni ha price me </t>
   </si>
   <si>
     <t xml:space="preserve">Total Component Cost </t>
@@ -1683,7 +1676,7 @@
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <numFmts count="3">
     <numFmt numFmtId="164" formatCode="[$-409]h:mm:ss\ AM/PM;@"/>
     <numFmt numFmtId="165" formatCode="&quot;$&quot;#,##0.0000"/>
@@ -2217,7 +2210,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="0" fontId="20" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="112">
+  <cellXfs count="106">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -2387,21 +2380,6 @@
     <xf numFmtId="0" fontId="20" fillId="4" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="18" fillId="6" borderId="17" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="20" fillId="6" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="21" fillId="2" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2436,9 +2414,6 @@
     <xf numFmtId="166" fontId="15" fillId="3" borderId="21" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="22" fillId="6" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="22" fillId="6" borderId="18" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2451,9 +2426,6 @@
     <xf numFmtId="0" fontId="23" fillId="6" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="6" borderId="17" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="25" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -2490,14 +2462,14 @@
     <xf numFmtId="0" fontId="18" fillId="4" borderId="25" xfId="0" quotePrefix="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="6" borderId="25" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="18" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="6" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="3" borderId="22" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1" applyProtection="1">
       <alignment horizontal="center" vertical="top"/>
@@ -2531,8 +2503,11 @@
     <xf numFmtId="0" fontId="17" fillId="3" borderId="20" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="18" fillId="2" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="0" fontId="20" fillId="2" borderId="17" xfId="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="4" borderId="19" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -2578,7 +2553,7 @@
         <xdr:cNvPr id="2" name="Picture 1">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{00000000-0008-0000-0000-000002000000}"/>
+              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" xmlns="" id="{00000000-0008-0000-0000-000002000000}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -2874,7 +2849,7 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <sheetPr codeName="Sheet1"/>
   <dimension ref="A1:T104"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
@@ -2916,15 +2891,15 @@
       <c r="H1" s="2"/>
       <c r="I1" s="2"/>
       <c r="J1" s="2"/>
-      <c r="K1" s="103"/>
-      <c r="L1" s="103"/>
-      <c r="M1" s="103"/>
-      <c r="N1" s="103"/>
-      <c r="O1" s="103"/>
-      <c r="P1" s="103"/>
-      <c r="Q1" s="103"/>
-      <c r="R1" s="103"/>
-      <c r="S1" s="104"/>
+      <c r="K1" s="96"/>
+      <c r="L1" s="96"/>
+      <c r="M1" s="96"/>
+      <c r="N1" s="96"/>
+      <c r="O1" s="96"/>
+      <c r="P1" s="96"/>
+      <c r="Q1" s="96"/>
+      <c r="R1" s="96"/>
+      <c r="S1" s="97"/>
     </row>
     <row r="2" spans="1:19" ht="32.25" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A2" s="1"/>
@@ -2935,7 +2910,7 @@
       </c>
       <c r="E2" s="11"/>
       <c r="F2" s="54" t="s">
-        <v>524</v>
+        <v>522</v>
       </c>
       <c r="G2" s="12"/>
       <c r="H2" s="12"/>
@@ -2960,7 +2935,7 @@
       </c>
       <c r="E3" s="13"/>
       <c r="F3" s="55" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
       <c r="G3" s="13"/>
       <c r="H3" s="13"/>
@@ -2974,7 +2949,7 @@
       <c r="P3" s="5"/>
       <c r="Q3" s="5"/>
       <c r="R3" s="5"/>
-      <c r="S3" s="105"/>
+      <c r="S3" s="98"/>
     </row>
     <row r="4" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A4" s="1"/>
@@ -2985,7 +2960,7 @@
       </c>
       <c r="E4" s="13"/>
       <c r="F4" s="56" t="s">
-        <v>525</v>
+        <v>523</v>
       </c>
       <c r="G4" s="14"/>
       <c r="H4" s="14"/>
@@ -2999,7 +2974,7 @@
       <c r="P4" s="6"/>
       <c r="Q4" s="6"/>
       <c r="R4" s="6"/>
-      <c r="S4" s="106"/>
+      <c r="S4" s="99"/>
     </row>
     <row r="5" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A5" s="1"/>
@@ -3024,7 +2999,7 @@
       <c r="P5" s="6"/>
       <c r="Q5" s="6"/>
       <c r="R5" s="6"/>
-      <c r="S5" s="106"/>
+      <c r="S5" s="99"/>
     </row>
     <row r="6" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A6" s="1"/>
@@ -3045,7 +3020,7 @@
       <c r="P6" s="6"/>
       <c r="Q6" s="6"/>
       <c r="R6" s="6"/>
-      <c r="S6" s="106"/>
+      <c r="S6" s="99"/>
     </row>
     <row r="7" spans="1:19" x14ac:dyDescent="0.25">
       <c r="A7" s="1"/>
@@ -3066,7 +3041,7 @@
       <c r="P7" s="8"/>
       <c r="Q7" s="8"/>
       <c r="R7" s="8"/>
-      <c r="S7" s="106"/>
+      <c r="S7" s="99"/>
     </row>
     <row r="8" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="1"/>
@@ -3087,7 +3062,7 @@
       <c r="P8" s="8"/>
       <c r="Q8" s="8"/>
       <c r="R8" s="8"/>
-      <c r="S8" s="106"/>
+      <c r="S8" s="99"/>
     </row>
     <row r="9" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="1"/>
@@ -3118,7 +3093,7 @@
       <c r="J9" s="30" t="s">
         <v>400</v>
       </c>
-      <c r="K9" s="92" t="s">
+      <c r="K9" s="85" t="s">
         <v>412</v>
       </c>
       <c r="L9" s="30" t="s">
@@ -3152,7 +3127,7 @@
         <f t="shared" ref="B10:B41" si="0">ROW(B10) - ROW($B$9)</f>
         <v>1</v>
       </c>
-      <c r="C10" s="82" t="s">
+      <c r="C10" s="76" t="s">
         <v>385</v>
       </c>
       <c r="D10" s="46" t="s">
@@ -3176,7 +3151,7 @@
       <c r="J10" s="46" t="s">
         <v>413</v>
       </c>
-      <c r="K10" s="93" t="s">
+      <c r="K10" s="86" t="s">
         <v>338</v>
       </c>
       <c r="L10" s="46">
@@ -3208,7 +3183,7 @@
         <f t="shared" si="0"/>
         <v>2</v>
       </c>
-      <c r="C11" s="83" t="s">
+      <c r="C11" s="77" t="s">
         <v>385</v>
       </c>
       <c r="D11" s="50" t="s">
@@ -3232,7 +3207,7 @@
       <c r="J11" s="50" t="s">
         <v>415</v>
       </c>
-      <c r="K11" s="94" t="s">
+      <c r="K11" s="87" t="s">
         <v>339</v>
       </c>
       <c r="L11" s="50">
@@ -3264,7 +3239,7 @@
         <f t="shared" si="0"/>
         <v>3</v>
       </c>
-      <c r="C12" s="82" t="s">
+      <c r="C12" s="76" t="s">
         <v>385</v>
       </c>
       <c r="D12" s="46" t="s">
@@ -3288,7 +3263,7 @@
       <c r="J12" s="46" t="s">
         <v>416</v>
       </c>
-      <c r="K12" s="95" t="s">
+      <c r="K12" s="88" t="s">
         <v>340</v>
       </c>
       <c r="L12" s="46">
@@ -3320,7 +3295,7 @@
         <f t="shared" si="0"/>
         <v>4</v>
       </c>
-      <c r="C13" s="83" t="s">
+      <c r="C13" s="77" t="s">
         <v>385</v>
       </c>
       <c r="D13" s="50" t="s">
@@ -3344,7 +3319,7 @@
       <c r="J13" s="50" t="s">
         <v>417</v>
       </c>
-      <c r="K13" s="94" t="s">
+      <c r="K13" s="87" t="s">
         <v>341</v>
       </c>
       <c r="L13" s="50">
@@ -3376,7 +3351,7 @@
         <f t="shared" si="0"/>
         <v>5</v>
       </c>
-      <c r="C14" s="82" t="s">
+      <c r="C14" s="76" t="s">
         <v>385</v>
       </c>
       <c r="D14" s="46" t="s">
@@ -3400,7 +3375,7 @@
       <c r="J14" s="46" t="s">
         <v>418</v>
       </c>
-      <c r="K14" s="95" t="s">
+      <c r="K14" s="88" t="s">
         <v>342</v>
       </c>
       <c r="L14" s="46">
@@ -3423,8 +3398,8 @@
         <f t="shared" si="2"/>
         <v>1.3759999999999999</v>
       </c>
-      <c r="R14" s="81" t="s">
-        <v>539</v>
+      <c r="R14" s="75" t="s">
+        <v>537</v>
       </c>
       <c r="S14" s="48"/>
     </row>
@@ -3434,7 +3409,7 @@
         <f t="shared" si="0"/>
         <v>6</v>
       </c>
-      <c r="C15" s="83" t="s">
+      <c r="C15" s="77" t="s">
         <v>385</v>
       </c>
       <c r="D15" s="50" t="s">
@@ -3458,7 +3433,7 @@
       <c r="J15" s="50" t="s">
         <v>419</v>
       </c>
-      <c r="K15" s="94" t="s">
+      <c r="K15" s="87" t="s">
         <v>343</v>
       </c>
       <c r="L15" s="50">
@@ -3490,58 +3465,58 @@
         <f t="shared" si="0"/>
         <v>7</v>
       </c>
-      <c r="C16" s="84" t="s">
+      <c r="C16" s="78" t="s">
         <v>385</v>
       </c>
-      <c r="D16" s="73" t="s">
+      <c r="D16" s="68" t="s">
         <v>13</v>
       </c>
-      <c r="E16" s="74" t="s">
+      <c r="E16" s="69" t="s">
         <v>105</v>
       </c>
-      <c r="F16" s="73" t="s">
+      <c r="F16" s="68" t="s">
         <v>408</v>
       </c>
-      <c r="G16" s="100" t="s">
+      <c r="G16" s="92" t="s">
         <v>193</v>
       </c>
-      <c r="H16" s="73" t="s">
-        <v>526</v>
-      </c>
-      <c r="I16" s="73" t="s">
+      <c r="H16" s="68" t="s">
+        <v>524</v>
+      </c>
+      <c r="I16" s="68" t="s">
         <v>301</v>
       </c>
-      <c r="J16" s="73" t="s">
-        <v>527</v>
-      </c>
-      <c r="K16" s="96" t="s">
+      <c r="J16" s="68" t="s">
+        <v>525</v>
+      </c>
+      <c r="K16" s="89" t="s">
         <v>340</v>
       </c>
-      <c r="L16" s="73">
+      <c r="L16" s="68">
         <v>1</v>
       </c>
-      <c r="M16" s="73">
+      <c r="M16" s="68">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="N16" s="73">
+      <c r="N16" s="68">
         <v>10</v>
       </c>
-      <c r="O16" s="89" t="s">
-        <v>414</v>
-      </c>
-      <c r="P16" s="75">
+      <c r="O16" s="82" t="s">
+        <v>414</v>
+      </c>
+      <c r="P16" s="70">
         <v>0.187</v>
       </c>
-      <c r="Q16" s="75">
+      <c r="Q16" s="70">
         <f t="shared" si="2"/>
         <v>1.87</v>
       </c>
-      <c r="R16" s="81" t="s">
-        <v>538</v>
-      </c>
-      <c r="S16" s="76" t="s">
-        <v>528</v>
+      <c r="R16" s="75" t="s">
+        <v>536</v>
+      </c>
+      <c r="S16" s="71" t="s">
+        <v>526</v>
       </c>
     </row>
     <row r="17" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -3550,7 +3525,7 @@
         <f t="shared" si="0"/>
         <v>8</v>
       </c>
-      <c r="C17" s="83" t="s">
+      <c r="C17" s="77" t="s">
         <v>385</v>
       </c>
       <c r="D17" s="50" t="s">
@@ -3574,7 +3549,7 @@
       <c r="J17" s="50" t="s">
         <v>420</v>
       </c>
-      <c r="K17" s="94" t="s">
+      <c r="K17" s="87" t="s">
         <v>344</v>
       </c>
       <c r="L17" s="50">
@@ -3606,7 +3581,7 @@
         <f t="shared" si="0"/>
         <v>9</v>
       </c>
-      <c r="C18" s="82" t="s">
+      <c r="C18" s="76" t="s">
         <v>385</v>
       </c>
       <c r="D18" s="46" t="s">
@@ -3630,7 +3605,7 @@
       <c r="J18" s="46" t="s">
         <v>421</v>
       </c>
-      <c r="K18" s="95" t="s">
+      <c r="K18" s="88" t="s">
         <v>345</v>
       </c>
       <c r="L18" s="46">
@@ -3662,7 +3637,7 @@
         <f t="shared" si="0"/>
         <v>10</v>
       </c>
-      <c r="C19" s="83" t="s">
+      <c r="C19" s="77" t="s">
         <v>385</v>
       </c>
       <c r="D19" s="50" t="s">
@@ -3686,7 +3661,7 @@
       <c r="J19" s="50" t="s">
         <v>422</v>
       </c>
-      <c r="K19" s="94" t="s">
+      <c r="K19" s="87" t="s">
         <v>339</v>
       </c>
       <c r="L19" s="50">
@@ -3718,7 +3693,7 @@
         <f t="shared" si="0"/>
         <v>11</v>
       </c>
-      <c r="C20" s="82" t="s">
+      <c r="C20" s="76" t="s">
         <v>385</v>
       </c>
       <c r="D20" s="46" t="s">
@@ -3742,7 +3717,7 @@
       <c r="J20" s="46" t="s">
         <v>423</v>
       </c>
-      <c r="K20" s="95" t="s">
+      <c r="K20" s="88" t="s">
         <v>346</v>
       </c>
       <c r="L20" s="46">
@@ -3774,7 +3749,7 @@
         <f t="shared" si="0"/>
         <v>12</v>
       </c>
-      <c r="C21" s="83" t="s">
+      <c r="C21" s="77" t="s">
         <v>385</v>
       </c>
       <c r="D21" s="50" t="s">
@@ -3798,7 +3773,7 @@
       <c r="J21" s="50" t="s">
         <v>424</v>
       </c>
-      <c r="K21" s="94" t="s">
+      <c r="K21" s="87" t="s">
         <v>347</v>
       </c>
       <c r="L21" s="50">
@@ -3830,7 +3805,7 @@
         <f t="shared" si="0"/>
         <v>13</v>
       </c>
-      <c r="C22" s="82" t="s">
+      <c r="C22" s="76" t="s">
         <v>385</v>
       </c>
       <c r="D22" s="46" t="s">
@@ -3854,7 +3829,7 @@
       <c r="J22" s="46" t="s">
         <v>425</v>
       </c>
-      <c r="K22" s="95" t="s">
+      <c r="K22" s="88" t="s">
         <v>348</v>
       </c>
       <c r="L22" s="46">
@@ -3886,7 +3861,7 @@
         <f t="shared" si="0"/>
         <v>14</v>
       </c>
-      <c r="C23" s="83" t="s">
+      <c r="C23" s="77" t="s">
         <v>385</v>
       </c>
       <c r="D23" s="50" t="s">
@@ -3910,7 +3885,7 @@
       <c r="J23" s="50" t="s">
         <v>426</v>
       </c>
-      <c r="K23" s="94" t="s">
+      <c r="K23" s="87" t="s">
         <v>349</v>
       </c>
       <c r="L23" s="50">
@@ -3942,7 +3917,7 @@
         <f t="shared" si="0"/>
         <v>15</v>
       </c>
-      <c r="C24" s="82" t="s">
+      <c r="C24" s="76" t="s">
         <v>385</v>
       </c>
       <c r="D24" s="46" t="s">
@@ -3954,7 +3929,7 @@
       <c r="F24" s="46" t="s">
         <v>190</v>
       </c>
-      <c r="G24" s="68" t="s">
+      <c r="G24" s="63" t="s">
         <v>248</v>
       </c>
       <c r="H24" s="46" t="s">
@@ -3966,7 +3941,7 @@
       <c r="J24" s="46" t="s">
         <v>475</v>
       </c>
-      <c r="K24" s="95" t="s">
+      <c r="K24" s="88" t="s">
         <v>350</v>
       </c>
       <c r="L24" s="46">
@@ -3998,7 +3973,7 @@
         <f t="shared" si="0"/>
         <v>16</v>
       </c>
-      <c r="C25" s="83" t="s">
+      <c r="C25" s="77" t="s">
         <v>385</v>
       </c>
       <c r="D25" s="50" t="s">
@@ -4010,19 +3985,19 @@
       <c r="F25" s="50" t="s">
         <v>190</v>
       </c>
-      <c r="G25" s="69" t="s">
+      <c r="G25" s="64" t="s">
         <v>249</v>
       </c>
       <c r="H25" s="50" t="s">
-        <v>540</v>
+        <v>538</v>
       </c>
       <c r="I25" s="50" t="s">
         <v>298</v>
       </c>
       <c r="J25" s="50" t="s">
-        <v>541</v>
-      </c>
-      <c r="K25" s="94" t="s">
+        <v>539</v>
+      </c>
+      <c r="K25" s="87" t="s">
         <v>351</v>
       </c>
       <c r="L25" s="50">
@@ -4054,7 +4029,7 @@
         <f t="shared" si="0"/>
         <v>17</v>
       </c>
-      <c r="C26" s="82" t="s">
+      <c r="C26" s="76" t="s">
         <v>386</v>
       </c>
       <c r="D26" s="46" t="s">
@@ -4078,7 +4053,7 @@
       <c r="J26" s="46" t="s">
         <v>476</v>
       </c>
-      <c r="K26" s="95" t="s">
+      <c r="K26" s="88" t="s">
         <v>410</v>
       </c>
       <c r="L26" s="46">
@@ -4110,7 +4085,7 @@
         <f t="shared" si="0"/>
         <v>18</v>
       </c>
-      <c r="C27" s="83" t="s">
+      <c r="C27" s="77" t="s">
         <v>386</v>
       </c>
       <c r="D27" s="50" t="s">
@@ -4134,7 +4109,7 @@
       <c r="J27" s="50" t="s">
         <v>427</v>
       </c>
-      <c r="K27" s="94" t="s">
+      <c r="K27" s="87" t="s">
         <v>410</v>
       </c>
       <c r="L27" s="50">
@@ -4166,7 +4141,7 @@
         <f t="shared" si="0"/>
         <v>19</v>
       </c>
-      <c r="C28" s="82" t="s">
+      <c r="C28" s="76" t="s">
         <v>386</v>
       </c>
       <c r="D28" s="46" t="s">
@@ -4190,7 +4165,7 @@
       <c r="J28" s="46" t="s">
         <v>479</v>
       </c>
-      <c r="K28" s="95" t="s">
+      <c r="K28" s="88" t="s">
         <v>410</v>
       </c>
       <c r="L28" s="46">
@@ -4222,7 +4197,7 @@
         <f t="shared" si="0"/>
         <v>20</v>
       </c>
-      <c r="C29" s="83" t="s">
+      <c r="C29" s="77" t="s">
         <v>386</v>
       </c>
       <c r="D29" s="50" t="s">
@@ -4246,7 +4221,7 @@
       <c r="J29" s="50" t="s">
         <v>428</v>
       </c>
-      <c r="K29" s="94" t="s">
+      <c r="K29" s="87" t="s">
         <v>410</v>
       </c>
       <c r="L29" s="50">
@@ -4278,58 +4253,58 @@
         <f t="shared" si="0"/>
         <v>21</v>
       </c>
-      <c r="C30" s="84" t="s">
+      <c r="C30" s="78" t="s">
         <v>386</v>
       </c>
-      <c r="D30" s="73" t="s">
+      <c r="D30" s="68" t="s">
         <v>27</v>
       </c>
-      <c r="E30" s="74" t="s">
+      <c r="E30" s="69" t="s">
         <v>119</v>
       </c>
-      <c r="F30" s="73" t="s">
+      <c r="F30" s="68" t="s">
         <v>196</v>
       </c>
-      <c r="G30" s="100" t="s">
+      <c r="G30" s="92" t="s">
         <v>252</v>
       </c>
-      <c r="H30" s="73" t="s">
-        <v>529</v>
-      </c>
-      <c r="I30" s="73" t="s">
+      <c r="H30" s="68" t="s">
+        <v>527</v>
+      </c>
+      <c r="I30" s="68" t="s">
         <v>305</v>
       </c>
-      <c r="J30" s="73" t="s">
-        <v>530</v>
-      </c>
-      <c r="K30" s="96" t="s">
-        <v>410</v>
-      </c>
-      <c r="L30" s="73">
+      <c r="J30" s="68" t="s">
+        <v>528</v>
+      </c>
+      <c r="K30" s="89" t="s">
+        <v>410</v>
+      </c>
+      <c r="L30" s="68">
         <v>1</v>
       </c>
-      <c r="M30" s="73">
+      <c r="M30" s="68">
         <f t="shared" si="1"/>
         <v>5</v>
       </c>
-      <c r="N30" s="73">
+      <c r="N30" s="68">
         <v>10</v>
       </c>
-      <c r="O30" s="89" t="s">
-        <v>414</v>
-      </c>
-      <c r="P30" s="75">
+      <c r="O30" s="82" t="s">
+        <v>414</v>
+      </c>
+      <c r="P30" s="70">
         <v>6.9000000000000006E-2</v>
       </c>
-      <c r="Q30" s="75">
+      <c r="Q30" s="70">
         <f t="shared" si="2"/>
         <v>0.69000000000000006</v>
       </c>
-      <c r="R30" s="81" t="s">
-        <v>538</v>
-      </c>
-      <c r="S30" s="76" t="s">
-        <v>531</v>
+      <c r="R30" s="75" t="s">
+        <v>536</v>
+      </c>
+      <c r="S30" s="71" t="s">
+        <v>529</v>
       </c>
     </row>
     <row r="31" spans="1:19" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -4338,7 +4313,7 @@
         <f t="shared" si="0"/>
         <v>22</v>
       </c>
-      <c r="C31" s="83" t="s">
+      <c r="C31" s="77" t="s">
         <v>386</v>
       </c>
       <c r="D31" s="50" t="s">
@@ -4362,7 +4337,7 @@
       <c r="J31" s="50" t="s">
         <v>481</v>
       </c>
-      <c r="K31" s="94" t="s">
+      <c r="K31" s="87" t="s">
         <v>410</v>
       </c>
       <c r="L31" s="50">
@@ -4394,7 +4369,7 @@
         <f t="shared" si="0"/>
         <v>23</v>
       </c>
-      <c r="C32" s="82" t="s">
+      <c r="C32" s="76" t="s">
         <v>387</v>
       </c>
       <c r="D32" s="46" t="s">
@@ -4414,7 +4389,7 @@
         <v>307</v>
       </c>
       <c r="J32" s="46"/>
-      <c r="K32" s="95" t="s">
+      <c r="K32" s="88" t="s">
         <v>410</v>
       </c>
       <c r="L32" s="46">
@@ -4440,7 +4415,7 @@
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="C33" s="83" t="s">
+      <c r="C33" s="77" t="s">
         <v>388</v>
       </c>
       <c r="D33" s="50" t="s">
@@ -4452,7 +4427,7 @@
       <c r="F33" s="50" t="s">
         <v>408</v>
       </c>
-      <c r="G33" s="69" t="s">
+      <c r="G33" s="64" t="s">
         <v>199</v>
       </c>
       <c r="H33" s="50" t="s">
@@ -4464,7 +4439,7 @@
       <c r="J33" s="50" t="s">
         <v>513</v>
       </c>
-      <c r="K33" s="94" t="s">
+      <c r="K33" s="87" t="s">
         <v>410</v>
       </c>
       <c r="L33" s="50">
@@ -4496,7 +4471,7 @@
         <f t="shared" si="0"/>
         <v>25</v>
       </c>
-      <c r="C34" s="82" t="s">
+      <c r="C34" s="76" t="s">
         <v>388</v>
       </c>
       <c r="D34" s="46" t="s">
@@ -4508,7 +4483,7 @@
       <c r="F34" s="46" t="s">
         <v>408</v>
       </c>
-      <c r="G34" s="68" t="s">
+      <c r="G34" s="63" t="s">
         <v>200</v>
       </c>
       <c r="H34" s="46" t="s">
@@ -4520,7 +4495,7 @@
       <c r="J34" s="46" t="s">
         <v>515</v>
       </c>
-      <c r="K34" s="95" t="s">
+      <c r="K34" s="88" t="s">
         <v>410</v>
       </c>
       <c r="L34" s="46">
@@ -4552,7 +4527,7 @@
         <f t="shared" si="0"/>
         <v>26</v>
       </c>
-      <c r="C35" s="83" t="s">
+      <c r="C35" s="77" t="s">
         <v>388</v>
       </c>
       <c r="D35" s="50" t="s">
@@ -4564,7 +4539,7 @@
       <c r="F35" s="50" t="s">
         <v>408</v>
       </c>
-      <c r="G35" s="69" t="s">
+      <c r="G35" s="64" t="s">
         <v>201</v>
       </c>
       <c r="H35" s="50" t="s">
@@ -4576,7 +4551,7 @@
       <c r="J35" s="50" t="s">
         <v>517</v>
       </c>
-      <c r="K35" s="97" t="s">
+      <c r="K35" s="90" t="s">
         <v>411</v>
       </c>
       <c r="L35" s="50">
@@ -4608,7 +4583,7 @@
         <f t="shared" si="0"/>
         <v>27</v>
       </c>
-      <c r="C36" s="82" t="s">
+      <c r="C36" s="76" t="s">
         <v>387</v>
       </c>
       <c r="D36" s="46" t="s">
@@ -4632,7 +4607,7 @@
       <c r="J36" s="46" t="s">
         <v>429</v>
       </c>
-      <c r="K36" s="95" t="s">
+      <c r="K36" s="88" t="s">
         <v>410</v>
       </c>
       <c r="L36" s="46">
@@ -4664,7 +4639,7 @@
         <f t="shared" si="0"/>
         <v>28</v>
       </c>
-      <c r="C37" s="83" t="s">
+      <c r="C37" s="77" t="s">
         <v>389</v>
       </c>
       <c r="D37" s="50" t="s">
@@ -4688,7 +4663,7 @@
       <c r="J37" s="50" t="s">
         <v>430</v>
       </c>
-      <c r="K37" s="94" t="s">
+      <c r="K37" s="87" t="s">
         <v>410</v>
       </c>
       <c r="L37" s="50">
@@ -4720,7 +4695,7 @@
         <f t="shared" si="0"/>
         <v>29</v>
       </c>
-      <c r="C38" s="82" t="s">
+      <c r="C38" s="76" t="s">
         <v>387</v>
       </c>
       <c r="D38" s="46" t="s">
@@ -4744,7 +4719,7 @@
       <c r="J38" s="46" t="s">
         <v>431</v>
       </c>
-      <c r="K38" s="95" t="s">
+      <c r="K38" s="88" t="s">
         <v>410</v>
       </c>
       <c r="L38" s="46">
@@ -4776,7 +4751,7 @@
         <f t="shared" si="0"/>
         <v>30</v>
       </c>
-      <c r="C39" s="83" t="s">
+      <c r="C39" s="77" t="s">
         <v>390</v>
       </c>
       <c r="D39" s="50" t="s">
@@ -4800,7 +4775,7 @@
       <c r="J39" s="50" t="s">
         <v>483</v>
       </c>
-      <c r="K39" s="94" t="s">
+      <c r="K39" s="87" t="s">
         <v>353</v>
       </c>
       <c r="L39" s="50">
@@ -4832,7 +4807,7 @@
         <f t="shared" si="0"/>
         <v>31</v>
       </c>
-      <c r="C40" s="82" t="s">
+      <c r="C40" s="76" t="s">
         <v>390</v>
       </c>
       <c r="D40" s="46" t="s">
@@ -4856,7 +4831,7 @@
       <c r="J40" s="46" t="s">
         <v>432</v>
       </c>
-      <c r="K40" s="95" t="s">
+      <c r="K40" s="88" t="s">
         <v>354</v>
       </c>
       <c r="L40" s="46">
@@ -4888,7 +4863,7 @@
         <f t="shared" si="0"/>
         <v>32</v>
       </c>
-      <c r="C41" s="83" t="s">
+      <c r="C41" s="77" t="s">
         <v>390</v>
       </c>
       <c r="D41" s="50" t="s">
@@ -4912,7 +4887,7 @@
       <c r="J41" s="50" t="s">
         <v>433</v>
       </c>
-      <c r="K41" s="94" t="s">
+      <c r="K41" s="87" t="s">
         <v>355</v>
       </c>
       <c r="L41" s="50">
@@ -4944,7 +4919,7 @@
         <f t="shared" ref="B42:B73" si="3">ROW(B42) - ROW($B$9)</f>
         <v>33</v>
       </c>
-      <c r="C42" s="82" t="s">
+      <c r="C42" s="76" t="s">
         <v>390</v>
       </c>
       <c r="D42" s="46" t="s">
@@ -4968,7 +4943,7 @@
       <c r="J42" s="46" t="s">
         <v>434</v>
       </c>
-      <c r="K42" s="95" t="s">
+      <c r="K42" s="88" t="s">
         <v>356</v>
       </c>
       <c r="L42" s="46">
@@ -5000,7 +4975,7 @@
         <f t="shared" si="3"/>
         <v>34</v>
       </c>
-      <c r="C43" s="83" t="s">
+      <c r="C43" s="77" t="s">
         <v>391</v>
       </c>
       <c r="D43" s="50" t="s">
@@ -5012,7 +4987,7 @@
       <c r="F43" s="50" t="s">
         <v>209</v>
       </c>
-      <c r="G43" s="69" t="s">
+      <c r="G43" s="64" t="s">
         <v>255</v>
       </c>
       <c r="H43" s="50" t="s">
@@ -5024,7 +4999,7 @@
       <c r="J43" s="50" t="s">
         <v>500</v>
       </c>
-      <c r="K43" s="94" t="s">
+      <c r="K43" s="87" t="s">
         <v>410</v>
       </c>
       <c r="L43" s="50">
@@ -5056,7 +5031,7 @@
         <f t="shared" si="3"/>
         <v>35</v>
       </c>
-      <c r="C44" s="82" t="s">
+      <c r="C44" s="76" t="s">
         <v>391</v>
       </c>
       <c r="D44" s="46" t="s">
@@ -5080,7 +5055,7 @@
       <c r="J44" s="46" t="s">
         <v>435</v>
       </c>
-      <c r="K44" s="95" t="s">
+      <c r="K44" s="88" t="s">
         <v>410</v>
       </c>
       <c r="L44" s="46">
@@ -5112,7 +5087,7 @@
         <f t="shared" si="3"/>
         <v>36</v>
       </c>
-      <c r="C45" s="83" t="s">
+      <c r="C45" s="77" t="s">
         <v>392</v>
       </c>
       <c r="D45" s="50" t="s">
@@ -5136,7 +5111,7 @@
       <c r="J45" s="50" t="s">
         <v>436</v>
       </c>
-      <c r="K45" s="94" t="s">
+      <c r="K45" s="87" t="s">
         <v>410</v>
       </c>
       <c r="L45" s="50">
@@ -5168,7 +5143,7 @@
         <f t="shared" si="3"/>
         <v>37</v>
       </c>
-      <c r="C46" s="82" t="s">
+      <c r="C46" s="76" t="s">
         <v>357</v>
       </c>
       <c r="D46" s="46" t="s">
@@ -5192,7 +5167,7 @@
       <c r="J46" s="46" t="s">
         <v>410</v>
       </c>
-      <c r="K46" s="95" t="s">
+      <c r="K46" s="88" t="s">
         <v>410</v>
       </c>
       <c r="L46" s="46">
@@ -5214,8 +5189,8 @@
       <c r="Q46" s="60" t="s">
         <v>410</v>
       </c>
-      <c r="R46" s="87" t="s">
-        <v>523</v>
+      <c r="R46" s="80" t="s">
+        <v>521</v>
       </c>
       <c r="S46" s="48" t="s">
         <v>410</v>
@@ -5227,7 +5202,7 @@
         <f t="shared" si="3"/>
         <v>38</v>
       </c>
-      <c r="C47" s="83" t="s">
+      <c r="C47" s="77" t="s">
         <v>389</v>
       </c>
       <c r="D47" s="50" t="s">
@@ -5239,7 +5214,7 @@
       <c r="F47" s="50" t="s">
         <v>211</v>
       </c>
-      <c r="G47" s="69">
+      <c r="G47" s="64">
         <v>61300311121</v>
       </c>
       <c r="H47" s="50" t="s">
@@ -5251,7 +5226,7 @@
       <c r="J47" s="50" t="s">
         <v>487</v>
       </c>
-      <c r="K47" s="94" t="s">
+      <c r="K47" s="87" t="s">
         <v>410</v>
       </c>
       <c r="L47" s="50">
@@ -5283,7 +5258,7 @@
         <f t="shared" si="3"/>
         <v>39</v>
       </c>
-      <c r="C48" s="82" t="s">
+      <c r="C48" s="76" t="s">
         <v>389</v>
       </c>
       <c r="D48" s="46" t="s">
@@ -5295,7 +5270,7 @@
       <c r="F48" s="46" t="s">
         <v>212</v>
       </c>
-      <c r="G48" s="68">
+      <c r="G48" s="63">
         <v>61300611121</v>
       </c>
       <c r="H48" s="46" t="s">
@@ -5307,7 +5282,7 @@
       <c r="J48" s="46" t="s">
         <v>485</v>
       </c>
-      <c r="K48" s="95" t="s">
+      <c r="K48" s="88" t="s">
         <v>410</v>
       </c>
       <c r="L48" s="46">
@@ -5339,7 +5314,7 @@
         <f t="shared" si="3"/>
         <v>40</v>
       </c>
-      <c r="C49" s="83" t="s">
+      <c r="C49" s="77" t="s">
         <v>389</v>
       </c>
       <c r="D49" s="50" t="s">
@@ -5351,7 +5326,7 @@
       <c r="F49" s="50" t="s">
         <v>213</v>
       </c>
-      <c r="G49" s="69" t="s">
+      <c r="G49" s="64" t="s">
         <v>257</v>
       </c>
       <c r="H49" s="50" t="s">
@@ -5363,7 +5338,7 @@
       <c r="J49" s="50" t="s">
         <v>501</v>
       </c>
-      <c r="K49" s="94" t="s">
+      <c r="K49" s="87" t="s">
         <v>410</v>
       </c>
       <c r="L49" s="50">
@@ -5395,7 +5370,7 @@
         <f t="shared" si="3"/>
         <v>41</v>
       </c>
-      <c r="C50" s="82" t="s">
+      <c r="C50" s="76" t="s">
         <v>389</v>
       </c>
       <c r="D50" s="46" t="s">
@@ -5407,19 +5382,19 @@
       <c r="F50" s="46" t="s">
         <v>214</v>
       </c>
-      <c r="G50" s="68">
+      <c r="G50" s="63">
         <v>61300211121</v>
       </c>
-      <c r="H50" s="111" t="s">
-        <v>542</v>
+      <c r="H50" s="93" t="s">
+        <v>540</v>
       </c>
       <c r="I50" s="46" t="s">
         <v>319</v>
       </c>
       <c r="J50" s="46" t="s">
-        <v>543</v>
-      </c>
-      <c r="K50" s="95" t="s">
+        <v>541</v>
+      </c>
+      <c r="K50" s="88" t="s">
         <v>410</v>
       </c>
       <c r="L50" s="46">
@@ -5451,7 +5426,7 @@
         <f t="shared" si="3"/>
         <v>42</v>
       </c>
-      <c r="C51" s="83" t="s">
+      <c r="C51" s="77" t="s">
         <v>389</v>
       </c>
       <c r="D51" s="50" t="s">
@@ -5463,7 +5438,7 @@
       <c r="F51" s="50" t="s">
         <v>215</v>
       </c>
-      <c r="G51" s="69">
+      <c r="G51" s="64">
         <v>61300411121</v>
       </c>
       <c r="H51" s="50" t="s">
@@ -5475,7 +5450,7 @@
       <c r="J51" s="50" t="s">
         <v>489</v>
       </c>
-      <c r="K51" s="94" t="s">
+      <c r="K51" s="87" t="s">
         <v>410</v>
       </c>
       <c r="L51" s="50">
@@ -5507,7 +5482,7 @@
         <f t="shared" si="3"/>
         <v>43</v>
       </c>
-      <c r="C52" s="82" t="s">
+      <c r="C52" s="76" t="s">
         <v>393</v>
       </c>
       <c r="D52" s="46" t="s">
@@ -5531,7 +5506,7 @@
       <c r="J52" s="46" t="s">
         <v>437</v>
       </c>
-      <c r="K52" s="95" t="s">
+      <c r="K52" s="88" t="s">
         <v>410</v>
       </c>
       <c r="L52" s="46">
@@ -5563,7 +5538,7 @@
         <f t="shared" si="3"/>
         <v>44</v>
       </c>
-      <c r="C53" s="83" t="s">
+      <c r="C53" s="77" t="s">
         <v>393</v>
       </c>
       <c r="D53" s="50" t="s">
@@ -5587,7 +5562,7 @@
       <c r="J53" s="50" t="s">
         <v>491</v>
       </c>
-      <c r="K53" s="94" t="s">
+      <c r="K53" s="87" t="s">
         <v>410</v>
       </c>
       <c r="L53" s="50">
@@ -5619,7 +5594,7 @@
         <f t="shared" si="3"/>
         <v>45</v>
       </c>
-      <c r="C54" s="82" t="s">
+      <c r="C54" s="76" t="s">
         <v>393</v>
       </c>
       <c r="D54" s="46" t="s">
@@ -5643,7 +5618,7 @@
       <c r="J54" s="46" t="s">
         <v>438</v>
       </c>
-      <c r="K54" s="95" t="s">
+      <c r="K54" s="88" t="s">
         <v>410</v>
       </c>
       <c r="L54" s="46">
@@ -5675,7 +5650,7 @@
         <f t="shared" si="3"/>
         <v>46</v>
       </c>
-      <c r="C55" s="83" t="s">
+      <c r="C55" s="77" t="s">
         <v>393</v>
       </c>
       <c r="D55" s="50" t="s">
@@ -5687,7 +5662,7 @@
       <c r="F55" s="50" t="s">
         <v>217</v>
       </c>
-      <c r="G55" s="70" t="s">
+      <c r="G55" s="65" t="s">
         <v>261</v>
       </c>
       <c r="H55" s="50" t="s">
@@ -5699,7 +5674,7 @@
       <c r="J55" s="50" t="s">
         <v>492</v>
       </c>
-      <c r="K55" s="94" t="s">
+      <c r="K55" s="87" t="s">
         <v>410</v>
       </c>
       <c r="L55" s="50">
@@ -5731,7 +5706,7 @@
         <f t="shared" si="3"/>
         <v>47</v>
       </c>
-      <c r="C56" s="82" t="s">
+      <c r="C56" s="76" t="s">
         <v>393</v>
       </c>
       <c r="D56" s="46" t="s">
@@ -5753,7 +5728,7 @@
       <c r="J56" s="46" t="s">
         <v>439</v>
       </c>
-      <c r="K56" s="95" t="s">
+      <c r="K56" s="88" t="s">
         <v>410</v>
       </c>
       <c r="L56" s="46">
@@ -5785,7 +5760,7 @@
         <f t="shared" si="3"/>
         <v>48</v>
       </c>
-      <c r="C57" s="83" t="s">
+      <c r="C57" s="77" t="s">
         <v>393</v>
       </c>
       <c r="D57" s="50" t="s">
@@ -5809,7 +5784,7 @@
       <c r="J57" s="50" t="s">
         <v>440</v>
       </c>
-      <c r="K57" s="94" t="s">
+      <c r="K57" s="87" t="s">
         <v>410</v>
       </c>
       <c r="L57" s="50">
@@ -5841,7 +5816,7 @@
         <f t="shared" si="3"/>
         <v>49</v>
       </c>
-      <c r="C58" s="82" t="s">
+      <c r="C58" s="76" t="s">
         <v>393</v>
       </c>
       <c r="D58" s="46" t="s">
@@ -5865,7 +5840,7 @@
       <c r="J58" s="46" t="s">
         <v>441</v>
       </c>
-      <c r="K58" s="95" t="s">
+      <c r="K58" s="88" t="s">
         <v>410</v>
       </c>
       <c r="L58" s="46">
@@ -5897,7 +5872,7 @@
         <f t="shared" si="3"/>
         <v>50</v>
       </c>
-      <c r="C59" s="83" t="s">
+      <c r="C59" s="77" t="s">
         <v>393</v>
       </c>
       <c r="D59" s="50" t="s">
@@ -5921,7 +5896,7 @@
       <c r="J59" s="50" t="s">
         <v>442</v>
       </c>
-      <c r="K59" s="94" t="s">
+      <c r="K59" s="87" t="s">
         <v>410</v>
       </c>
       <c r="L59" s="50">
@@ -5953,7 +5928,7 @@
         <f t="shared" si="3"/>
         <v>51</v>
       </c>
-      <c r="C60" s="82" t="s">
+      <c r="C60" s="76" t="s">
         <v>394</v>
       </c>
       <c r="D60" s="46" t="s">
@@ -5963,7 +5938,7 @@
         <v>147</v>
       </c>
       <c r="F60" s="46" t="s">
-        <v>544</v>
+        <v>542</v>
       </c>
       <c r="G60" s="47" t="s">
         <v>265</v>
@@ -5977,7 +5952,7 @@
       <c r="J60" s="46" t="s">
         <v>443</v>
       </c>
-      <c r="K60" s="95" t="s">
+      <c r="K60" s="88" t="s">
         <v>358</v>
       </c>
       <c r="L60" s="46">
@@ -6009,7 +5984,7 @@
         <f t="shared" si="3"/>
         <v>52</v>
       </c>
-      <c r="C61" s="83" t="s">
+      <c r="C61" s="77" t="s">
         <v>394</v>
       </c>
       <c r="D61" s="50" t="s">
@@ -6031,7 +6006,7 @@
       <c r="J61" s="50" t="s">
         <v>444</v>
       </c>
-      <c r="K61" s="94" t="s">
+      <c r="K61" s="87" t="s">
         <v>359</v>
       </c>
       <c r="L61" s="50">
@@ -6063,7 +6038,7 @@
         <f t="shared" si="3"/>
         <v>53</v>
       </c>
-      <c r="C62" s="82" t="s">
+      <c r="C62" s="76" t="s">
         <v>394</v>
       </c>
       <c r="D62" s="46" t="s">
@@ -6087,7 +6062,7 @@
       <c r="J62" s="46" t="s">
         <v>473</v>
       </c>
-      <c r="K62" s="95" t="s">
+      <c r="K62" s="88" t="s">
         <v>360</v>
       </c>
       <c r="L62" s="46">
@@ -6119,11 +6094,11 @@
         <f t="shared" si="3"/>
         <v>54</v>
       </c>
-      <c r="C63" s="83" t="s">
+      <c r="C63" s="77" t="s">
         <v>394</v>
       </c>
       <c r="D63" s="50" t="s">
-        <v>537</v>
+        <v>535</v>
       </c>
       <c r="E63" s="51" t="s">
         <v>150</v>
@@ -6143,7 +6118,7 @@
       <c r="J63" s="50" t="s">
         <v>445</v>
       </c>
-      <c r="K63" s="94" t="s">
+      <c r="K63" s="87" t="s">
         <v>361</v>
       </c>
       <c r="L63" s="50">
@@ -6175,7 +6150,7 @@
         <f t="shared" si="3"/>
         <v>55</v>
       </c>
-      <c r="C64" s="82" t="s">
+      <c r="C64" s="76" t="s">
         <v>394</v>
       </c>
       <c r="D64" s="46" t="s">
@@ -6199,7 +6174,7 @@
       <c r="J64" s="46" t="s">
         <v>446</v>
       </c>
-      <c r="K64" s="95" t="s">
+      <c r="K64" s="88" t="s">
         <v>362</v>
       </c>
       <c r="L64" s="46">
@@ -6231,7 +6206,7 @@
         <f t="shared" si="3"/>
         <v>56</v>
       </c>
-      <c r="C65" s="83" t="s">
+      <c r="C65" s="77" t="s">
         <v>394</v>
       </c>
       <c r="D65" s="50" t="s">
@@ -6253,7 +6228,7 @@
       <c r="J65" s="50" t="s">
         <v>447</v>
       </c>
-      <c r="K65" s="94" t="s">
+      <c r="K65" s="87" t="s">
         <v>363</v>
       </c>
       <c r="L65" s="50">
@@ -6285,7 +6260,7 @@
         <f t="shared" si="3"/>
         <v>57</v>
       </c>
-      <c r="C66" s="82" t="s">
+      <c r="C66" s="76" t="s">
         <v>394</v>
       </c>
       <c r="D66" s="46" t="s">
@@ -6309,7 +6284,7 @@
       <c r="J66" s="46" t="s">
         <v>448</v>
       </c>
-      <c r="K66" s="95" t="s">
+      <c r="K66" s="88" t="s">
         <v>364</v>
       </c>
       <c r="L66" s="46">
@@ -6341,7 +6316,7 @@
         <f t="shared" si="3"/>
         <v>58</v>
       </c>
-      <c r="C67" s="83" t="s">
+      <c r="C67" s="77" t="s">
         <v>394</v>
       </c>
       <c r="D67" s="50" t="s">
@@ -6353,7 +6328,7 @@
       <c r="F67" s="50" t="s">
         <v>220</v>
       </c>
-      <c r="G67" s="69" t="s">
+      <c r="G67" s="64" t="s">
         <v>271</v>
       </c>
       <c r="H67" s="50" t="s">
@@ -6365,7 +6340,7 @@
       <c r="J67" s="50" t="s">
         <v>494</v>
       </c>
-      <c r="K67" s="94" t="s">
+      <c r="K67" s="87" t="s">
         <v>365</v>
       </c>
       <c r="L67" s="50">
@@ -6397,7 +6372,7 @@
         <f t="shared" si="3"/>
         <v>59</v>
       </c>
-      <c r="C68" s="82" t="s">
+      <c r="C68" s="76" t="s">
         <v>394</v>
       </c>
       <c r="D68" s="46" t="s">
@@ -6421,7 +6396,7 @@
       <c r="J68" s="46" t="s">
         <v>449</v>
       </c>
-      <c r="K68" s="95" t="s">
+      <c r="K68" s="88" t="s">
         <v>366</v>
       </c>
       <c r="L68" s="46">
@@ -6453,7 +6428,7 @@
         <f t="shared" si="3"/>
         <v>60</v>
       </c>
-      <c r="C69" s="83" t="s">
+      <c r="C69" s="77" t="s">
         <v>394</v>
       </c>
       <c r="D69" s="50" t="s">
@@ -6477,7 +6452,7 @@
       <c r="J69" s="50" t="s">
         <v>450</v>
       </c>
-      <c r="K69" s="94" t="s">
+      <c r="K69" s="87" t="s">
         <v>367</v>
       </c>
       <c r="L69" s="50">
@@ -6509,7 +6484,7 @@
         <f t="shared" si="3"/>
         <v>61</v>
       </c>
-      <c r="C70" s="82" t="s">
+      <c r="C70" s="76" t="s">
         <v>394</v>
       </c>
       <c r="D70" s="46" t="s">
@@ -6533,7 +6508,7 @@
       <c r="J70" s="46" t="s">
         <v>451</v>
       </c>
-      <c r="K70" s="95" t="s">
+      <c r="K70" s="88" t="s">
         <v>368</v>
       </c>
       <c r="L70" s="46">
@@ -6565,7 +6540,7 @@
         <f t="shared" si="3"/>
         <v>62</v>
       </c>
-      <c r="C71" s="83" t="s">
+      <c r="C71" s="77" t="s">
         <v>394</v>
       </c>
       <c r="D71" s="50" t="s">
@@ -6589,7 +6564,7 @@
       <c r="J71" s="50" t="s">
         <v>452</v>
       </c>
-      <c r="K71" s="94" t="s">
+      <c r="K71" s="87" t="s">
         <v>369</v>
       </c>
       <c r="L71" s="50">
@@ -6621,7 +6596,7 @@
         <f t="shared" si="3"/>
         <v>63</v>
       </c>
-      <c r="C72" s="82" t="s">
+      <c r="C72" s="76" t="s">
         <v>394</v>
       </c>
       <c r="D72" s="46" t="s">
@@ -6645,7 +6620,7 @@
       <c r="J72" s="46" t="s">
         <v>453</v>
       </c>
-      <c r="K72" s="95" t="s">
+      <c r="K72" s="88" t="s">
         <v>370</v>
       </c>
       <c r="L72" s="46">
@@ -6677,7 +6652,7 @@
         <f t="shared" si="3"/>
         <v>64</v>
       </c>
-      <c r="C73" s="83" t="s">
+      <c r="C73" s="77" t="s">
         <v>394</v>
       </c>
       <c r="D73" s="50" t="s">
@@ -6701,7 +6676,7 @@
       <c r="J73" s="50" t="s">
         <v>454</v>
       </c>
-      <c r="K73" s="94" t="s">
+      <c r="K73" s="87" t="s">
         <v>371</v>
       </c>
       <c r="L73" s="50">
@@ -6733,7 +6708,7 @@
         <f t="shared" ref="B74:B101" si="4">ROW(B74) - ROW($B$9)</f>
         <v>65</v>
       </c>
-      <c r="C74" s="82" t="s">
+      <c r="C74" s="76" t="s">
         <v>394</v>
       </c>
       <c r="D74" s="46" t="s">
@@ -6757,7 +6732,7 @@
       <c r="J74" s="46" t="s">
         <v>506</v>
       </c>
-      <c r="K74" s="95" t="s">
+      <c r="K74" s="88" t="s">
         <v>503</v>
       </c>
       <c r="L74" s="46">
@@ -6780,7 +6755,7 @@
         <f t="shared" si="2"/>
         <v>0.16</v>
       </c>
-      <c r="R74" s="88"/>
+      <c r="R74" s="81"/>
       <c r="S74" s="48"/>
     </row>
     <row r="75" spans="1:19" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -6789,7 +6764,7 @@
         <f t="shared" si="4"/>
         <v>66</v>
       </c>
-      <c r="C75" s="83" t="s">
+      <c r="C75" s="77" t="s">
         <v>394</v>
       </c>
       <c r="D75" s="50" t="s">
@@ -6813,7 +6788,7 @@
       <c r="J75" s="50" t="s">
         <v>455</v>
       </c>
-      <c r="K75" s="94" t="s">
+      <c r="K75" s="87" t="s">
         <v>372</v>
       </c>
       <c r="L75" s="50">
@@ -6845,7 +6820,7 @@
         <f t="shared" si="4"/>
         <v>67</v>
       </c>
-      <c r="C76" s="82" t="s">
+      <c r="C76" s="76" t="s">
         <v>394</v>
       </c>
       <c r="D76" s="46" t="s">
@@ -6869,7 +6844,7 @@
       <c r="J76" s="46" t="s">
         <v>456</v>
       </c>
-      <c r="K76" s="95" t="s">
+      <c r="K76" s="88" t="s">
         <v>373</v>
       </c>
       <c r="L76" s="46">
@@ -6901,7 +6876,7 @@
         <f t="shared" si="4"/>
         <v>68</v>
       </c>
-      <c r="C77" s="83" t="s">
+      <c r="C77" s="77" t="s">
         <v>394</v>
       </c>
       <c r="D77" s="50" t="s">
@@ -6925,7 +6900,7 @@
       <c r="J77" s="50" t="s">
         <v>457</v>
       </c>
-      <c r="K77" s="94" t="s">
+      <c r="K77" s="87" t="s">
         <v>374</v>
       </c>
       <c r="L77" s="50">
@@ -6957,7 +6932,7 @@
         <f t="shared" si="4"/>
         <v>69</v>
       </c>
-      <c r="C78" s="82" t="s">
+      <c r="C78" s="76" t="s">
         <v>394</v>
       </c>
       <c r="D78" s="46" t="s">
@@ -6969,7 +6944,7 @@
       <c r="F78" s="46" t="s">
         <v>221</v>
       </c>
-      <c r="G78" s="68" t="s">
+      <c r="G78" s="63" t="s">
         <v>281</v>
       </c>
       <c r="H78" s="46" t="s">
@@ -6981,7 +6956,7 @@
       <c r="J78" s="46" t="s">
         <v>508</v>
       </c>
-      <c r="K78" s="95" t="s">
+      <c r="K78" s="88" t="s">
         <v>375</v>
       </c>
       <c r="L78" s="46">
@@ -7013,7 +6988,7 @@
         <f t="shared" si="4"/>
         <v>70</v>
       </c>
-      <c r="C79" s="83" t="s">
+      <c r="C79" s="77" t="s">
         <v>394</v>
       </c>
       <c r="D79" s="50" t="s">
@@ -7037,7 +7012,7 @@
       <c r="J79" s="50" t="s">
         <v>458</v>
       </c>
-      <c r="K79" s="94" t="s">
+      <c r="K79" s="87" t="s">
         <v>376</v>
       </c>
       <c r="L79" s="50">
@@ -7069,7 +7044,7 @@
         <f t="shared" si="4"/>
         <v>71</v>
       </c>
-      <c r="C80" s="82" t="s">
+      <c r="C80" s="76" t="s">
         <v>394</v>
       </c>
       <c r="D80" s="46" t="s">
@@ -7093,7 +7068,7 @@
       <c r="J80" s="46" t="s">
         <v>459</v>
       </c>
-      <c r="K80" s="95" t="s">
+      <c r="K80" s="88" t="s">
         <v>377</v>
       </c>
       <c r="L80" s="46">
@@ -7125,7 +7100,7 @@
         <f t="shared" si="4"/>
         <v>72</v>
       </c>
-      <c r="C81" s="82" t="s">
+      <c r="C81" s="76" t="s">
         <v>394</v>
       </c>
       <c r="D81" s="46" t="s">
@@ -7149,7 +7124,7 @@
       <c r="J81" s="46" t="s">
         <v>460</v>
       </c>
-      <c r="K81" s="95" t="s">
+      <c r="K81" s="88" t="s">
         <v>378</v>
       </c>
       <c r="L81" s="46">
@@ -7181,7 +7156,7 @@
         <f t="shared" si="4"/>
         <v>73</v>
       </c>
-      <c r="C82" s="83" t="s">
+      <c r="C82" s="77" t="s">
         <v>394</v>
       </c>
       <c r="D82" s="50" t="s">
@@ -7205,7 +7180,7 @@
       <c r="J82" s="50" t="s">
         <v>461</v>
       </c>
-      <c r="K82" s="94" t="s">
+      <c r="K82" s="87" t="s">
         <v>379</v>
       </c>
       <c r="L82" s="50">
@@ -7237,7 +7212,7 @@
         <f t="shared" si="4"/>
         <v>74</v>
       </c>
-      <c r="C83" s="82" t="s">
+      <c r="C83" s="76" t="s">
         <v>394</v>
       </c>
       <c r="D83" s="46" t="s">
@@ -7261,7 +7236,7 @@
       <c r="J83" s="46" t="s">
         <v>496</v>
       </c>
-      <c r="K83" s="95" t="s">
+      <c r="K83" s="88" t="s">
         <v>380</v>
       </c>
       <c r="L83" s="46">
@@ -7293,7 +7268,7 @@
         <f t="shared" si="4"/>
         <v>75</v>
       </c>
-      <c r="C84" s="83" t="s">
+      <c r="C84" s="77" t="s">
         <v>394</v>
       </c>
       <c r="D84" s="50" t="s">
@@ -7317,7 +7292,7 @@
       <c r="J84" s="50" t="s">
         <v>462</v>
       </c>
-      <c r="K84" s="94" t="s">
+      <c r="K84" s="87" t="s">
         <v>381</v>
       </c>
       <c r="L84" s="50">
@@ -7349,7 +7324,7 @@
         <f t="shared" si="4"/>
         <v>76</v>
       </c>
-      <c r="C85" s="82" t="s">
+      <c r="C85" s="76" t="s">
         <v>394</v>
       </c>
       <c r="D85" s="46" t="s">
@@ -7361,7 +7336,7 @@
       <c r="F85" s="46" t="s">
         <v>223</v>
       </c>
-      <c r="G85" s="68" t="s">
+      <c r="G85" s="63" t="s">
         <v>287</v>
       </c>
       <c r="H85" s="46" t="s">
@@ -7373,7 +7348,7 @@
       <c r="J85" s="46" t="s">
         <v>498</v>
       </c>
-      <c r="K85" s="95" t="s">
+      <c r="K85" s="88" t="s">
         <v>362</v>
       </c>
       <c r="L85" s="46">
@@ -7405,7 +7380,7 @@
         <f t="shared" si="4"/>
         <v>77</v>
       </c>
-      <c r="C86" s="83" t="s">
+      <c r="C86" s="77" t="s">
         <v>224</v>
       </c>
       <c r="D86" s="50" t="s">
@@ -7429,7 +7404,7 @@
       <c r="J86" s="50" t="s">
         <v>410</v>
       </c>
-      <c r="K86" s="94" t="s">
+      <c r="K86" s="87" t="s">
         <v>410</v>
       </c>
       <c r="L86" s="50">
@@ -7439,22 +7414,22 @@
         <f t="shared" si="5"/>
         <v>90</v>
       </c>
-      <c r="N86" s="71" t="s">
-        <v>410</v>
-      </c>
-      <c r="O86" s="72" t="s">
-        <v>410</v>
-      </c>
-      <c r="P86" s="71" t="s">
-        <v>410</v>
-      </c>
-      <c r="Q86" s="72" t="s">
-        <v>410</v>
-      </c>
-      <c r="R86" s="86" t="s">
-        <v>523</v>
-      </c>
-      <c r="S86" s="72" t="s">
+      <c r="N86" s="66" t="s">
+        <v>410</v>
+      </c>
+      <c r="O86" s="67" t="s">
+        <v>410</v>
+      </c>
+      <c r="P86" s="66" t="s">
+        <v>410</v>
+      </c>
+      <c r="Q86" s="67" t="s">
+        <v>410</v>
+      </c>
+      <c r="R86" s="79" t="s">
+        <v>521</v>
+      </c>
+      <c r="S86" s="67" t="s">
         <v>410</v>
       </c>
     </row>
@@ -7464,7 +7439,7 @@
         <f t="shared" si="4"/>
         <v>78</v>
       </c>
-      <c r="C87" s="82" t="s">
+      <c r="C87" s="76" t="s">
         <v>395</v>
       </c>
       <c r="D87" s="46" t="s">
@@ -7488,7 +7463,7 @@
       <c r="J87" s="46" t="s">
         <v>463</v>
       </c>
-      <c r="K87" s="95" t="s">
+      <c r="K87" s="88" t="s">
         <v>410</v>
       </c>
       <c r="L87" s="46">
@@ -7514,64 +7489,62 @@
       <c r="R87" s="48"/>
       <c r="S87" s="48"/>
     </row>
-    <row r="88" spans="1:20" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:20" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A88" s="1"/>
       <c r="B88" s="38">
         <f t="shared" si="4"/>
         <v>79</v>
       </c>
-      <c r="C88" s="85" t="s">
+      <c r="C88" s="77" t="s">
         <v>396</v>
       </c>
-      <c r="D88" s="63" t="s">
+      <c r="D88" s="50" t="s">
         <v>84</v>
       </c>
-      <c r="E88" s="64" t="s">
+      <c r="E88" s="51" t="s">
         <v>175</v>
       </c>
-      <c r="F88" s="63" t="s">
+      <c r="F88" s="50" t="s">
         <v>226</v>
       </c>
-      <c r="G88" s="64" t="s">
+      <c r="G88" s="51" t="s">
         <v>288</v>
       </c>
-      <c r="H88" s="63" t="s">
-        <v>410</v>
-      </c>
-      <c r="I88" s="63" t="s">
+      <c r="H88" s="50" t="s">
+        <v>410</v>
+      </c>
+      <c r="I88" s="50" t="s">
         <v>331</v>
       </c>
-      <c r="J88" s="63" t="s">
-        <v>410</v>
-      </c>
-      <c r="K88" s="98" t="s">
-        <v>410</v>
-      </c>
-      <c r="L88" s="63">
+      <c r="J88" s="50" t="s">
+        <v>410</v>
+      </c>
+      <c r="K88" s="87" t="s">
+        <v>410</v>
+      </c>
+      <c r="L88" s="50">
         <v>2</v>
       </c>
-      <c r="M88" s="63">
+      <c r="M88" s="50">
         <f t="shared" si="5"/>
         <v>10</v>
       </c>
-      <c r="N88" s="63">
-        <v>10</v>
-      </c>
-      <c r="O88" s="67" t="s">
-        <v>518</v>
-      </c>
-      <c r="P88" s="65">
-        <v>8</v>
-      </c>
-      <c r="Q88" s="65">
+      <c r="N88" s="50">
+        <v>12</v>
+      </c>
+      <c r="O88" s="62" t="s">
+        <v>408</v>
+      </c>
+      <c r="P88" s="61">
+        <v>10.59</v>
+      </c>
+      <c r="Q88" s="61">
         <f t="shared" si="6"/>
-        <v>80</v>
-      </c>
-      <c r="R88" s="80" t="s">
-        <v>519</v>
-      </c>
-      <c r="S88" s="66"/>
-      <c r="T88" s="77"/>
+        <v>127.08</v>
+      </c>
+      <c r="R88" s="105"/>
+      <c r="S88" s="52"/>
+      <c r="T88" s="72"/>
     </row>
     <row r="89" spans="1:20" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A89" s="1"/>
@@ -7579,7 +7552,7 @@
         <f t="shared" si="4"/>
         <v>80</v>
       </c>
-      <c r="C89" s="82" t="s">
+      <c r="C89" s="76" t="s">
         <v>396</v>
       </c>
       <c r="D89" s="46" t="s">
@@ -7603,7 +7576,7 @@
       <c r="J89" s="46" t="s">
         <v>509</v>
       </c>
-      <c r="K89" s="95" t="s">
+      <c r="K89" s="88" t="s">
         <v>410</v>
       </c>
       <c r="L89" s="46">
@@ -7635,7 +7608,7 @@
         <f t="shared" si="4"/>
         <v>81</v>
       </c>
-      <c r="C90" s="83" t="s">
+      <c r="C90" s="77" t="s">
         <v>396</v>
       </c>
       <c r="D90" s="50" t="s">
@@ -7659,7 +7632,7 @@
       <c r="J90" s="50" t="s">
         <v>464</v>
       </c>
-      <c r="K90" s="94" t="s">
+      <c r="K90" s="87" t="s">
         <v>410</v>
       </c>
       <c r="L90" s="50">
@@ -7691,7 +7664,7 @@
         <f t="shared" si="4"/>
         <v>82</v>
       </c>
-      <c r="C91" s="82" t="s">
+      <c r="C91" s="76" t="s">
         <v>396</v>
       </c>
       <c r="D91" s="46" t="s">
@@ -7715,7 +7688,7 @@
       <c r="J91" s="46" t="s">
         <v>465</v>
       </c>
-      <c r="K91" s="95" t="s">
+      <c r="K91" s="88" t="s">
         <v>410</v>
       </c>
       <c r="L91" s="46">
@@ -7747,49 +7720,53 @@
         <f t="shared" si="4"/>
         <v>83</v>
       </c>
-      <c r="C92" s="85" t="s">
+      <c r="C92" s="77" t="s">
         <v>396</v>
       </c>
-      <c r="D92" s="63" t="s">
+      <c r="D92" s="50" t="s">
         <v>88</v>
       </c>
-      <c r="E92" s="64" t="s">
+      <c r="E92" s="51" t="s">
         <v>179</v>
       </c>
-      <c r="F92" s="63" t="s">
+      <c r="F92" s="50" t="s">
         <v>226</v>
       </c>
-      <c r="G92" s="64" t="s">
+      <c r="G92" s="51" t="s">
         <v>292</v>
       </c>
-      <c r="H92" s="63" t="s">
-        <v>410</v>
-      </c>
-      <c r="I92" s="63" t="s">
+      <c r="H92" s="50" t="s">
+        <v>410</v>
+      </c>
+      <c r="I92" s="50" t="s">
         <v>304</v>
       </c>
-      <c r="J92" s="63"/>
-      <c r="K92" s="98" t="s">
-        <v>410</v>
-      </c>
-      <c r="L92" s="63">
+      <c r="J92" s="50"/>
+      <c r="K92" s="87" t="s">
+        <v>410</v>
+      </c>
+      <c r="L92" s="50">
         <v>1</v>
       </c>
-      <c r="M92" s="63">
+      <c r="M92" s="50">
         <f t="shared" si="5"/>
         <v>5</v>
       </c>
-      <c r="N92" s="63">
+      <c r="N92" s="50">
         <v>6</v>
       </c>
-      <c r="O92" s="67"/>
-      <c r="P92" s="65"/>
-      <c r="Q92" s="65">
+      <c r="O92" s="62" t="s">
+        <v>408</v>
+      </c>
+      <c r="P92" s="61">
+        <v>1.48</v>
+      </c>
+      <c r="Q92" s="61">
         <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="R92" s="66"/>
-      <c r="S92" s="66"/>
+        <v>8.879999999999999</v>
+      </c>
+      <c r="R92" s="52"/>
+      <c r="S92" s="52"/>
     </row>
     <row r="93" spans="1:20" ht="24.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A93" s="1"/>
@@ -7797,47 +7774,53 @@
         <f t="shared" si="4"/>
         <v>84</v>
       </c>
-      <c r="C93" s="84" t="s">
+      <c r="C93" s="76" t="s">
         <v>396</v>
       </c>
-      <c r="D93" s="73" t="s">
+      <c r="D93" s="46" t="s">
         <v>89</v>
       </c>
-      <c r="E93" s="74" t="s">
+      <c r="E93" s="47" t="s">
         <v>180</v>
       </c>
-      <c r="F93" s="73" t="s">
+      <c r="F93" s="46" t="s">
         <v>409</v>
       </c>
-      <c r="G93" s="74" t="s">
+      <c r="G93" s="47" t="s">
         <v>229</v>
       </c>
-      <c r="H93" s="73" t="s">
-        <v>410</v>
-      </c>
-      <c r="I93" s="73" t="s">
+      <c r="H93" s="46" t="s">
+        <v>410</v>
+      </c>
+      <c r="I93" s="46" t="s">
         <v>334</v>
       </c>
-      <c r="J93" s="73"/>
-      <c r="K93" s="96" t="s">
-        <v>410</v>
-      </c>
-      <c r="L93" s="73">
+      <c r="J93" s="46"/>
+      <c r="K93" s="88" t="s">
+        <v>410</v>
+      </c>
+      <c r="L93" s="46">
         <v>1</v>
       </c>
-      <c r="M93" s="73">
+      <c r="M93" s="46">
         <f t="shared" si="5"/>
         <v>5</v>
       </c>
-      <c r="N93" s="73"/>
-      <c r="O93" s="73"/>
-      <c r="P93" s="75"/>
-      <c r="Q93" s="75">
+      <c r="N93" s="46">
+        <v>6</v>
+      </c>
+      <c r="O93" s="104" t="s">
+        <v>408</v>
+      </c>
+      <c r="P93" s="60">
+        <v>4.42</v>
+      </c>
+      <c r="Q93" s="60">
         <f t="shared" si="6"/>
-        <v>0</v>
-      </c>
-      <c r="R93" s="76"/>
-      <c r="S93" s="76"/>
+        <v>26.52</v>
+      </c>
+      <c r="R93" s="48"/>
+      <c r="S93" s="48"/>
     </row>
     <row r="94" spans="1:20" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A94" s="1"/>
@@ -7845,7 +7828,7 @@
         <f t="shared" si="4"/>
         <v>85</v>
       </c>
-      <c r="C94" s="83" t="s">
+      <c r="C94" s="77" t="s">
         <v>396</v>
       </c>
       <c r="D94" s="50" t="s">
@@ -7869,7 +7852,7 @@
       <c r="J94" s="50" t="s">
         <v>510</v>
       </c>
-      <c r="K94" s="94" t="s">
+      <c r="K94" s="87" t="s">
         <v>410</v>
       </c>
       <c r="L94" s="50">
@@ -7901,7 +7884,7 @@
         <f t="shared" si="4"/>
         <v>86</v>
       </c>
-      <c r="C95" s="82" t="s">
+      <c r="C95" s="76" t="s">
         <v>396</v>
       </c>
       <c r="D95" s="46" t="s">
@@ -7925,7 +7908,7 @@
       <c r="J95" s="46" t="s">
         <v>466</v>
       </c>
-      <c r="K95" s="95" t="s">
+      <c r="K95" s="88" t="s">
         <v>410</v>
       </c>
       <c r="L95" s="46">
@@ -7957,7 +7940,7 @@
         <f t="shared" si="4"/>
         <v>87</v>
       </c>
-      <c r="C96" s="83" t="s">
+      <c r="C96" s="77" t="s">
         <v>396</v>
       </c>
       <c r="D96" s="50" t="s">
@@ -7981,7 +7964,7 @@
       <c r="J96" s="50" t="s">
         <v>467</v>
       </c>
-      <c r="K96" s="94" t="s">
+      <c r="K96" s="87" t="s">
         <v>410</v>
       </c>
       <c r="L96" s="50">
@@ -8013,7 +7996,7 @@
         <f t="shared" si="4"/>
         <v>88</v>
       </c>
-      <c r="C97" s="82" t="s">
+      <c r="C97" s="76" t="s">
         <v>396</v>
       </c>
       <c r="D97" s="46" t="s">
@@ -8037,7 +8020,7 @@
       <c r="J97" s="46" t="s">
         <v>468</v>
       </c>
-      <c r="K97" s="95" t="s">
+      <c r="K97" s="88" t="s">
         <v>410</v>
       </c>
       <c r="L97" s="46">
@@ -8069,7 +8052,7 @@
         <f t="shared" si="4"/>
         <v>89</v>
       </c>
-      <c r="C98" s="83" t="s">
+      <c r="C98" s="77" t="s">
         <v>396</v>
       </c>
       <c r="D98" s="50" t="s">
@@ -8093,7 +8076,7 @@
       <c r="J98" s="50" t="s">
         <v>469</v>
       </c>
-      <c r="K98" s="94" t="s">
+      <c r="K98" s="87" t="s">
         <v>410</v>
       </c>
       <c r="L98" s="50">
@@ -8125,32 +8108,32 @@
         <f t="shared" si="4"/>
         <v>90</v>
       </c>
-      <c r="C99" s="82" t="s">
+      <c r="C99" s="76" t="s">
         <v>397</v>
       </c>
       <c r="D99" s="46" t="s">
         <v>95</v>
       </c>
       <c r="E99" s="47" t="s">
-        <v>535</v>
+        <v>533</v>
       </c>
       <c r="F99" s="46" t="s">
         <v>408</v>
       </c>
       <c r="G99" s="47" t="s">
+        <v>530</v>
+      </c>
+      <c r="H99" s="83" t="s">
+        <v>410</v>
+      </c>
+      <c r="I99" s="46" t="s">
+        <v>531</v>
+      </c>
+      <c r="J99" s="46" t="s">
+        <v>534</v>
+      </c>
+      <c r="K99" s="47" t="s">
         <v>532</v>
-      </c>
-      <c r="H99" s="90" t="s">
-        <v>410</v>
-      </c>
-      <c r="I99" s="46" t="s">
-        <v>533</v>
-      </c>
-      <c r="J99" s="46" t="s">
-        <v>536</v>
-      </c>
-      <c r="K99" s="47" t="s">
-        <v>534</v>
       </c>
       <c r="L99" s="46">
         <v>1</v>
@@ -8172,7 +8155,7 @@
         <f t="shared" si="6"/>
         <v>1.2804</v>
       </c>
-      <c r="R99" s="91"/>
+      <c r="R99" s="84"/>
       <c r="S99" s="48"/>
     </row>
     <row r="100" spans="1:19" ht="36.75" thickBot="1" x14ac:dyDescent="0.3">
@@ -8181,7 +8164,7 @@
         <f t="shared" si="4"/>
         <v>91</v>
       </c>
-      <c r="C100" s="83" t="s">
+      <c r="C100" s="77" t="s">
         <v>397</v>
       </c>
       <c r="D100" s="50" t="s">
@@ -8205,7 +8188,7 @@
       <c r="J100" s="50" t="s">
         <v>470</v>
       </c>
-      <c r="K100" s="94" t="s">
+      <c r="K100" s="87" t="s">
         <v>382</v>
       </c>
       <c r="L100" s="50">
@@ -8237,7 +8220,7 @@
         <f t="shared" si="4"/>
         <v>92</v>
       </c>
-      <c r="C101" s="82" t="s">
+      <c r="C101" s="76" t="s">
         <v>397</v>
       </c>
       <c r="D101" s="46" t="s">
@@ -8261,7 +8244,7 @@
       <c r="J101" s="46" t="s">
         <v>471</v>
       </c>
-      <c r="K101" s="99" t="s">
+      <c r="K101" s="91" t="s">
         <v>383</v>
       </c>
       <c r="L101" s="58">
@@ -8301,17 +8284,17 @@
       <c r="K102" s="37"/>
       <c r="L102" s="37"/>
       <c r="M102" s="37"/>
-      <c r="N102" s="101" t="s">
-        <v>520</v>
-      </c>
-      <c r="O102" s="102"/>
-      <c r="P102" s="102"/>
-      <c r="Q102" s="78">
+      <c r="N102" s="94" t="s">
+        <v>518</v>
+      </c>
+      <c r="O102" s="95"/>
+      <c r="P102" s="95"/>
+      <c r="Q102" s="73">
         <f>SUM(Q10:Q101)</f>
-        <v>634.95269999999994</v>
-      </c>
-      <c r="R102" s="107"/>
-      <c r="S102" s="108"/>
+        <v>717.43269999999995</v>
+      </c>
+      <c r="R102" s="100"/>
+      <c r="S102" s="101"/>
     </row>
     <row r="103" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A103" s="1"/>
@@ -8327,27 +8310,25 @@
       <c r="K103" s="10"/>
       <c r="L103" s="10"/>
       <c r="M103" s="10"/>
-      <c r="N103" s="101" t="s">
-        <v>521</v>
-      </c>
-      <c r="O103" s="102"/>
-      <c r="P103" s="102"/>
-      <c r="Q103" s="79">
+      <c r="N103" s="94" t="s">
+        <v>519</v>
+      </c>
+      <c r="O103" s="95"/>
+      <c r="P103" s="95"/>
+      <c r="Q103" s="74">
         <f>Q102/5</f>
-        <v>126.99053999999998</v>
-      </c>
-      <c r="R103" s="109"/>
-      <c r="S103" s="110"/>
+        <v>143.48653999999999</v>
+      </c>
+      <c r="R103" s="102"/>
+      <c r="S103" s="103"/>
     </row>
     <row r="104" spans="1:19" ht="19.5" thickBot="1" x14ac:dyDescent="0.3">
-      <c r="N104" s="101" t="s">
-        <v>522</v>
-      </c>
-      <c r="O104" s="102"/>
-      <c r="P104" s="102"/>
-      <c r="Q104" s="79">
-        <v>4</v>
-      </c>
+      <c r="N104" s="94" t="s">
+        <v>520</v>
+      </c>
+      <c r="O104" s="95"/>
+      <c r="P104" s="95"/>
+      <c r="Q104" s="74"/>
     </row>
   </sheetData>
   <mergeCells count="6">
@@ -8359,93 +8340,93 @@
     <mergeCell ref="N103:P103"/>
   </mergeCells>
   <hyperlinks>
-    <hyperlink ref="O10" r:id="rId1" xr:uid="{00000000-0004-0000-0000-000000000000}"/>
-    <hyperlink ref="O11" r:id="rId2" xr:uid="{00000000-0004-0000-0000-000001000000}"/>
-    <hyperlink ref="O12" r:id="rId3" xr:uid="{00000000-0004-0000-0000-000002000000}"/>
-    <hyperlink ref="O13" r:id="rId4" xr:uid="{00000000-0004-0000-0000-000003000000}"/>
-    <hyperlink ref="O14" r:id="rId5" xr:uid="{00000000-0004-0000-0000-000004000000}"/>
-    <hyperlink ref="O15" r:id="rId6" xr:uid="{00000000-0004-0000-0000-000005000000}"/>
-    <hyperlink ref="O17" r:id="rId7" xr:uid="{00000000-0004-0000-0000-000006000000}"/>
-    <hyperlink ref="O18" r:id="rId8" xr:uid="{00000000-0004-0000-0000-000007000000}"/>
-    <hyperlink ref="O19" r:id="rId9" xr:uid="{00000000-0004-0000-0000-000008000000}"/>
-    <hyperlink ref="O20" r:id="rId10" xr:uid="{00000000-0004-0000-0000-000009000000}"/>
-    <hyperlink ref="O21" r:id="rId11" xr:uid="{00000000-0004-0000-0000-00000A000000}"/>
-    <hyperlink ref="O22" r:id="rId12" xr:uid="{00000000-0004-0000-0000-00000B000000}"/>
-    <hyperlink ref="O23" r:id="rId13" xr:uid="{00000000-0004-0000-0000-00000C000000}"/>
-    <hyperlink ref="O27" r:id="rId14" xr:uid="{00000000-0004-0000-0000-00000E000000}"/>
-    <hyperlink ref="O36" r:id="rId15" xr:uid="{00000000-0004-0000-0000-00000F000000}"/>
-    <hyperlink ref="O37" r:id="rId16" xr:uid="{00000000-0004-0000-0000-000010000000}"/>
-    <hyperlink ref="O38" r:id="rId17" xr:uid="{00000000-0004-0000-0000-000011000000}"/>
-    <hyperlink ref="O40" r:id="rId18" xr:uid="{00000000-0004-0000-0000-000012000000}"/>
-    <hyperlink ref="O41" r:id="rId19" xr:uid="{00000000-0004-0000-0000-000013000000}"/>
-    <hyperlink ref="O42" r:id="rId20" xr:uid="{00000000-0004-0000-0000-000014000000}"/>
-    <hyperlink ref="O44" r:id="rId21" xr:uid="{00000000-0004-0000-0000-000015000000}"/>
-    <hyperlink ref="O45" r:id="rId22" xr:uid="{00000000-0004-0000-0000-000016000000}"/>
-    <hyperlink ref="O52" r:id="rId23" xr:uid="{00000000-0004-0000-0000-000017000000}"/>
-    <hyperlink ref="O54" r:id="rId24" xr:uid="{00000000-0004-0000-0000-000018000000}"/>
-    <hyperlink ref="O56" r:id="rId25" xr:uid="{00000000-0004-0000-0000-000019000000}"/>
-    <hyperlink ref="O57" r:id="rId26" xr:uid="{00000000-0004-0000-0000-00001A000000}"/>
-    <hyperlink ref="O58" r:id="rId27" xr:uid="{00000000-0004-0000-0000-00001B000000}"/>
-    <hyperlink ref="O59" r:id="rId28" xr:uid="{00000000-0004-0000-0000-00001C000000}"/>
-    <hyperlink ref="O60" r:id="rId29" xr:uid="{00000000-0004-0000-0000-00001D000000}"/>
-    <hyperlink ref="O61" r:id="rId30" xr:uid="{00000000-0004-0000-0000-00001E000000}"/>
-    <hyperlink ref="O62" r:id="rId31" xr:uid="{00000000-0004-0000-0000-00001F000000}"/>
-    <hyperlink ref="O63" r:id="rId32" xr:uid="{00000000-0004-0000-0000-000020000000}"/>
-    <hyperlink ref="O64" r:id="rId33" xr:uid="{00000000-0004-0000-0000-000021000000}"/>
-    <hyperlink ref="O65" r:id="rId34" xr:uid="{00000000-0004-0000-0000-000022000000}"/>
-    <hyperlink ref="O66" r:id="rId35" xr:uid="{00000000-0004-0000-0000-000023000000}"/>
-    <hyperlink ref="O68" r:id="rId36" xr:uid="{00000000-0004-0000-0000-000024000000}"/>
-    <hyperlink ref="O69" r:id="rId37" xr:uid="{00000000-0004-0000-0000-000025000000}"/>
-    <hyperlink ref="O70" r:id="rId38" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
-    <hyperlink ref="O71" r:id="rId39" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
-    <hyperlink ref="O72" r:id="rId40" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
-    <hyperlink ref="O73" r:id="rId41" xr:uid="{00000000-0004-0000-0000-000029000000}"/>
-    <hyperlink ref="O75" r:id="rId42" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
-    <hyperlink ref="O76" r:id="rId43" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
-    <hyperlink ref="O77" r:id="rId44" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
-    <hyperlink ref="O79" r:id="rId45" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
-    <hyperlink ref="O80" r:id="rId46" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
-    <hyperlink ref="O81" r:id="rId47" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
-    <hyperlink ref="O82" r:id="rId48" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
-    <hyperlink ref="O84" r:id="rId49" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
-    <hyperlink ref="O87" r:id="rId50" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
-    <hyperlink ref="O90" r:id="rId51" xr:uid="{00000000-0004-0000-0000-000033000000}"/>
-    <hyperlink ref="O91" r:id="rId52" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
-    <hyperlink ref="O95" r:id="rId53" xr:uid="{00000000-0004-0000-0000-000035000000}"/>
-    <hyperlink ref="O96" r:id="rId54" xr:uid="{00000000-0004-0000-0000-000036000000}"/>
-    <hyperlink ref="O97" r:id="rId55" xr:uid="{00000000-0004-0000-0000-000037000000}"/>
-    <hyperlink ref="O98" r:id="rId56" xr:uid="{00000000-0004-0000-0000-000038000000}"/>
-    <hyperlink ref="O100" r:id="rId57" xr:uid="{00000000-0004-0000-0000-000039000000}"/>
-    <hyperlink ref="O101" r:id="rId58" xr:uid="{00000000-0004-0000-0000-00003A000000}"/>
-    <hyperlink ref="O24" r:id="rId59" xr:uid="{00000000-0004-0000-0000-00003B000000}"/>
-    <hyperlink ref="O26" r:id="rId60" xr:uid="{00000000-0004-0000-0000-00003C000000}"/>
-    <hyperlink ref="O28" r:id="rId61" xr:uid="{00000000-0004-0000-0000-00003D000000}"/>
-    <hyperlink ref="O29" r:id="rId62" xr:uid="{00000000-0004-0000-0000-00003E000000}"/>
-    <hyperlink ref="O31" r:id="rId63" xr:uid="{00000000-0004-0000-0000-00003F000000}"/>
-    <hyperlink ref="O39" r:id="rId64" xr:uid="{00000000-0004-0000-0000-000040000000}"/>
-    <hyperlink ref="O48" r:id="rId65" xr:uid="{00000000-0004-0000-0000-000041000000}"/>
-    <hyperlink ref="O47" r:id="rId66" xr:uid="{00000000-0004-0000-0000-000042000000}"/>
-    <hyperlink ref="O51" r:id="rId67" xr:uid="{00000000-0004-0000-0000-000044000000}"/>
-    <hyperlink ref="O53" r:id="rId68" xr:uid="{00000000-0004-0000-0000-000045000000}"/>
-    <hyperlink ref="O55" r:id="rId69" xr:uid="{00000000-0004-0000-0000-000046000000}"/>
-    <hyperlink ref="O67" r:id="rId70" xr:uid="{00000000-0004-0000-0000-000047000000}"/>
-    <hyperlink ref="O83" r:id="rId71" xr:uid="{00000000-0004-0000-0000-000048000000}"/>
-    <hyperlink ref="O85" r:id="rId72" xr:uid="{00000000-0004-0000-0000-000049000000}"/>
-    <hyperlink ref="O43" r:id="rId73" xr:uid="{00000000-0004-0000-0000-00004A000000}"/>
-    <hyperlink ref="O49" r:id="rId74" xr:uid="{00000000-0004-0000-0000-00004B000000}"/>
-    <hyperlink ref="O74" r:id="rId75" xr:uid="{00000000-0004-0000-0000-00004C000000}"/>
-    <hyperlink ref="O78" r:id="rId76" xr:uid="{00000000-0004-0000-0000-00004D000000}"/>
-    <hyperlink ref="O89" r:id="rId77" xr:uid="{00000000-0004-0000-0000-00004E000000}"/>
-    <hyperlink ref="O94" r:id="rId78" xr:uid="{00000000-0004-0000-0000-00004F000000}"/>
-    <hyperlink ref="O33" r:id="rId79" xr:uid="{00000000-0004-0000-0000-000050000000}"/>
-    <hyperlink ref="O34" r:id="rId80" xr:uid="{00000000-0004-0000-0000-000051000000}"/>
-    <hyperlink ref="O35" r:id="rId81" xr:uid="{00000000-0004-0000-0000-000052000000}"/>
-    <hyperlink ref="O88" r:id="rId82" xr:uid="{00000000-0004-0000-0000-000053000000}"/>
-    <hyperlink ref="O16" r:id="rId83" xr:uid="{00000000-0004-0000-0000-000054000000}"/>
-    <hyperlink ref="O30" r:id="rId84" xr:uid="{00000000-0004-0000-0000-000055000000}"/>
-    <hyperlink ref="O99" r:id="rId85" xr:uid="{41DBDB4E-DF1C-471F-AD20-8FB2CA7D9E5E}"/>
-    <hyperlink ref="O25" r:id="rId86" xr:uid="{DAC6EF1B-A44F-4325-8C76-4CC4A05529DD}"/>
-    <hyperlink ref="O50" r:id="rId87" xr:uid="{249CEE1C-EC12-47D3-9B5F-AD078E9DD01C}"/>
+    <hyperlink ref="O10" r:id="rId1"/>
+    <hyperlink ref="O11" r:id="rId2"/>
+    <hyperlink ref="O12" r:id="rId3"/>
+    <hyperlink ref="O13" r:id="rId4"/>
+    <hyperlink ref="O14" r:id="rId5"/>
+    <hyperlink ref="O15" r:id="rId6"/>
+    <hyperlink ref="O17" r:id="rId7"/>
+    <hyperlink ref="O18" r:id="rId8"/>
+    <hyperlink ref="O19" r:id="rId9"/>
+    <hyperlink ref="O20" r:id="rId10"/>
+    <hyperlink ref="O21" r:id="rId11"/>
+    <hyperlink ref="O22" r:id="rId12"/>
+    <hyperlink ref="O23" r:id="rId13"/>
+    <hyperlink ref="O27" r:id="rId14"/>
+    <hyperlink ref="O36" r:id="rId15"/>
+    <hyperlink ref="O37" r:id="rId16"/>
+    <hyperlink ref="O38" r:id="rId17"/>
+    <hyperlink ref="O40" r:id="rId18"/>
+    <hyperlink ref="O41" r:id="rId19"/>
+    <hyperlink ref="O42" r:id="rId20"/>
+    <hyperlink ref="O44" r:id="rId21"/>
+    <hyperlink ref="O45" r:id="rId22"/>
+    <hyperlink ref="O52" r:id="rId23"/>
+    <hyperlink ref="O54" r:id="rId24"/>
+    <hyperlink ref="O56" r:id="rId25"/>
+    <hyperlink ref="O57" r:id="rId26"/>
+    <hyperlink ref="O58" r:id="rId27"/>
+    <hyperlink ref="O59" r:id="rId28"/>
+    <hyperlink ref="O60" r:id="rId29"/>
+    <hyperlink ref="O61" r:id="rId30"/>
+    <hyperlink ref="O62" r:id="rId31"/>
+    <hyperlink ref="O63" r:id="rId32"/>
+    <hyperlink ref="O64" r:id="rId33"/>
+    <hyperlink ref="O65" r:id="rId34"/>
+    <hyperlink ref="O66" r:id="rId35"/>
+    <hyperlink ref="O68" r:id="rId36"/>
+    <hyperlink ref="O69" r:id="rId37"/>
+    <hyperlink ref="O70" r:id="rId38"/>
+    <hyperlink ref="O71" r:id="rId39"/>
+    <hyperlink ref="O72" r:id="rId40"/>
+    <hyperlink ref="O73" r:id="rId41"/>
+    <hyperlink ref="O75" r:id="rId42"/>
+    <hyperlink ref="O76" r:id="rId43"/>
+    <hyperlink ref="O77" r:id="rId44"/>
+    <hyperlink ref="O79" r:id="rId45"/>
+    <hyperlink ref="O80" r:id="rId46"/>
+    <hyperlink ref="O81" r:id="rId47"/>
+    <hyperlink ref="O82" r:id="rId48"/>
+    <hyperlink ref="O84" r:id="rId49"/>
+    <hyperlink ref="O87" r:id="rId50"/>
+    <hyperlink ref="O90" r:id="rId51"/>
+    <hyperlink ref="O91" r:id="rId52"/>
+    <hyperlink ref="O95" r:id="rId53"/>
+    <hyperlink ref="O96" r:id="rId54"/>
+    <hyperlink ref="O97" r:id="rId55"/>
+    <hyperlink ref="O98" r:id="rId56"/>
+    <hyperlink ref="O100" r:id="rId57"/>
+    <hyperlink ref="O101" r:id="rId58"/>
+    <hyperlink ref="O24" r:id="rId59"/>
+    <hyperlink ref="O26" r:id="rId60"/>
+    <hyperlink ref="O28" r:id="rId61"/>
+    <hyperlink ref="O29" r:id="rId62"/>
+    <hyperlink ref="O31" r:id="rId63"/>
+    <hyperlink ref="O39" r:id="rId64"/>
+    <hyperlink ref="O48" r:id="rId65"/>
+    <hyperlink ref="O47" r:id="rId66"/>
+    <hyperlink ref="O51" r:id="rId67"/>
+    <hyperlink ref="O53" r:id="rId68"/>
+    <hyperlink ref="O55" r:id="rId69"/>
+    <hyperlink ref="O67" r:id="rId70"/>
+    <hyperlink ref="O83" r:id="rId71"/>
+    <hyperlink ref="O85" r:id="rId72"/>
+    <hyperlink ref="O43" r:id="rId73"/>
+    <hyperlink ref="O49" r:id="rId74"/>
+    <hyperlink ref="O74" r:id="rId75"/>
+    <hyperlink ref="O78" r:id="rId76"/>
+    <hyperlink ref="O89" r:id="rId77"/>
+    <hyperlink ref="O94" r:id="rId78"/>
+    <hyperlink ref="O33" r:id="rId79"/>
+    <hyperlink ref="O34" r:id="rId80"/>
+    <hyperlink ref="O35" r:id="rId81"/>
+    <hyperlink ref="O88" r:id="rId82" display="Aliexpress"/>
+    <hyperlink ref="O16" r:id="rId83"/>
+    <hyperlink ref="O30" r:id="rId84"/>
+    <hyperlink ref="O99" r:id="rId85"/>
+    <hyperlink ref="O25" r:id="rId86"/>
+    <hyperlink ref="O50" r:id="rId87"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId88"/>

</xml_diff>